<commit_message>
Split weekly wash reports by location
</commit_message>
<xml_diff>
--- a/backend/templates/report_template.xlsx
+++ b/backend/templates/report_template.xlsx
@@ -15,7 +15,8 @@
     <sheet name="ЦКР (Д)" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="ЦКР (Н)" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Мойка (Д)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Мойка (Н)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Мойка ул. Строителей (Н)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Мойка Ульяновская (Н)" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Арсенал (Д)'!$A$1:$I$26</definedName>
@@ -27,7 +28,6 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'ЦКР (Д)'!$A$1:$I$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'ЦКР (Н)'!$A$1:$I$39</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'Мойка (Д)'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Мойка (Н)'!$A$1:$I$31</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" refMode="R1C1"/>
 </workbook>
@@ -1748,6 +1748,490 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col width="1.42578125" customWidth="1" style="47" min="1" max="1"/>
+    <col width="34" customWidth="1" style="47" min="2" max="2"/>
+    <col width="2" customWidth="1" style="47" min="3" max="3"/>
+    <col width="13" customWidth="1" style="47" min="4" max="4"/>
+    <col width="2" customWidth="1" style="47" min="5" max="5"/>
+    <col width="13" customWidth="1" style="47" min="6" max="6"/>
+    <col width="2" customWidth="1" style="47" min="7" max="7"/>
+    <col width="13" customWidth="1" style="47" min="8" max="8"/>
+    <col width="14" customWidth="1" style="47" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="27.75" customHeight="1" s="47">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — МОЙКА</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1" s="47">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
+        </is>
+      </c>
+      <c r="B2" s="48" t="n"/>
+      <c r="C2" s="48" t="n"/>
+      <c r="D2" s="48" t="n"/>
+      <c r="E2" s="48" t="n"/>
+      <c r="F2" s="48" t="n"/>
+      <c r="G2" s="48" t="n"/>
+      <c r="H2" s="48" t="n"/>
+      <c r="I2" s="48" t="n"/>
+    </row>
+    <row r="3" ht="16.5" customHeight="1" s="47">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>АТЦ:</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="n"/>
+      <c r="E3" s="48" t="n"/>
+      <c r="F3" s="48" t="n"/>
+      <c r="G3" s="48" t="n"/>
+      <c r="H3" s="48" t="n"/>
+      <c r="I3" s="49" t="n"/>
+    </row>
+    <row r="4" ht="16.5" customHeight="1" s="47">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Неделя (авто):</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="n"/>
+      <c r="E4" s="48" t="n"/>
+      <c r="F4" s="48" t="n"/>
+      <c r="G4" s="48" t="n"/>
+      <c r="H4" s="48" t="n"/>
+      <c r="I4" s="49" t="n"/>
+    </row>
+    <row r="5" ht="16.5" customHeight="1" s="47">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Руководитель (авто):</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="n"/>
+      <c r="E5" s="48" t="n"/>
+      <c r="F5" s="48" t="n"/>
+      <c r="G5" s="48" t="n"/>
+      <c r="H5" s="48" t="n"/>
+      <c r="I5" s="49" t="n"/>
+    </row>
+    <row r="6" ht="6" customHeight="1" s="47"/>
+    <row r="7" ht="19.5" customHeight="1" s="47">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1.  КЛЮЧЕВЫЕ ПОКАЗАТЕЛИ  [из 1С]</t>
+        </is>
+      </c>
+      <c r="B7" s="50" t="n"/>
+      <c r="C7" s="50" t="n"/>
+      <c r="D7" s="50" t="n"/>
+      <c r="E7" s="50" t="n"/>
+      <c r="F7" s="50" t="n"/>
+      <c r="G7" s="50" t="n"/>
+      <c r="H7" s="50" t="n"/>
+      <c r="I7" s="50" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="47">
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>ПЛАН</t>
+        </is>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>ФАКТ (1С)</t>
+        </is>
+      </c>
+      <c r="H8" s="32" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I8" s="32" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18.75" customHeight="1" s="47">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Машин за неделю</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="n"/>
+      <c r="F9" s="28" t="n"/>
+      <c r="H9" s="6">
+        <f>IFERROR(IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9&gt;0),F9/D9,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18.75" customHeight="1" s="47">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Выручка за неделю</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="n"/>
+      <c r="F10" s="28" t="n"/>
+      <c r="H10" s="6">
+        <f>IFERROR(IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&gt;0),F10/D10,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18.75" customHeight="1" s="47">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Средний чек</t>
+        </is>
+      </c>
+      <c r="D11" s="8">
+        <f>IFERROR(D10/D9,"—")</f>
+        <v/>
+      </c>
+      <c r="F11" s="8">
+        <f>IFERROR(F10/F9,"—")</f>
+        <v/>
+      </c>
+      <c r="H11" s="6">
+        <f>IFERROR(IF(AND(ISNUMBER(D11),ISNUMBER(F11),D11&gt;0),F11/D11,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="6" customHeight="1" s="47"/>
+    <row r="13" ht="19.5" customHeight="1" s="47">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.  ДИНАМИКА ПО ДНЯМ  [из 1С]</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="n"/>
+      <c r="C13" s="50" t="n"/>
+      <c r="D13" s="50" t="n"/>
+      <c r="E13" s="50" t="n"/>
+      <c r="F13" s="50" t="n"/>
+      <c r="G13" s="50" t="n"/>
+      <c r="H13" s="50" t="n"/>
+      <c r="I13" s="50" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="47">
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>День</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>Машин</t>
+        </is>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>Выручка</t>
+        </is>
+      </c>
+      <c r="H14" s="32" t="inlineStr">
+        <is>
+          <t>Ср.чек</t>
+        </is>
+      </c>
+      <c r="I14" s="32" t="inlineStr">
+        <is>
+          <t>Операторов</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16.5" customHeight="1" s="47">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="n"/>
+      <c r="F15" s="28" t="n"/>
+      <c r="H15" s="8">
+        <f>IFERROR(F15/D15,"—")</f>
+        <v/>
+      </c>
+      <c r="I15" s="28" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1" s="47">
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="n"/>
+      <c r="F16" s="28" t="n"/>
+      <c r="H16" s="8">
+        <f>IFERROR(F16/D16,"—")</f>
+        <v/>
+      </c>
+      <c r="I16" s="28" t="n"/>
+    </row>
+    <row r="17" ht="16.5" customHeight="1" s="47">
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="n"/>
+      <c r="F17" s="28" t="n"/>
+      <c r="H17" s="8">
+        <f>IFERROR(F17/D17,"—")</f>
+        <v/>
+      </c>
+      <c r="I17" s="28" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1" s="47">
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="n"/>
+      <c r="F18" s="28" t="n"/>
+      <c r="H18" s="8">
+        <f>IFERROR(F18/D18,"—")</f>
+        <v/>
+      </c>
+      <c r="I18" s="28" t="n"/>
+    </row>
+    <row r="19" ht="16.5" customHeight="1" s="47">
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="D19" s="28" t="n"/>
+      <c r="F19" s="28" t="n"/>
+      <c r="H19" s="8">
+        <f>IFERROR(F19/D19,"—")</f>
+        <v/>
+      </c>
+      <c r="I19" s="28" t="n"/>
+    </row>
+    <row r="20" ht="16.5" customHeight="1" s="47">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Сб</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="n"/>
+      <c r="F20" s="28" t="n"/>
+      <c r="H20" s="8">
+        <f>IFERROR(F20/D20,"—")</f>
+        <v/>
+      </c>
+      <c r="I20" s="28" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1" s="47">
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Вс</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="n"/>
+      <c r="F21" s="28" t="n"/>
+      <c r="H21" s="8">
+        <f>IFERROR(F21/D21,"—")</f>
+        <v/>
+      </c>
+      <c r="I21" s="28" t="n"/>
+    </row>
+    <row r="22" ht="19.5" customHeight="1" s="47">
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="D22" s="11">
+        <f>SUM(D15:D21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="11">
+        <f>SUM(F15:F21)</f>
+        <v/>
+      </c>
+      <c r="H22" s="11">
+        <f>IFERROR(F22/D22,"—")</f>
+        <v/>
+      </c>
+      <c r="I22" s="15" t="n"/>
+    </row>
+    <row r="23" ht="6" customHeight="1" s="47"/>
+    <row r="24" ht="19.5" customHeight="1" s="47">
+      <c r="A24" s="36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3.  КОММЕНТАРИЙ РУКОВОДИТЕЛЯ  [вручную]</t>
+        </is>
+      </c>
+      <c r="B24" s="50" t="n"/>
+      <c r="C24" s="50" t="n"/>
+      <c r="D24" s="50" t="n"/>
+      <c r="E24" s="50" t="n"/>
+      <c r="F24" s="50" t="n"/>
+      <c r="G24" s="50" t="n"/>
+      <c r="H24" s="50" t="n"/>
+      <c r="I24" s="50" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="47">
+      <c r="B25" s="37" t="inlineStr">
+        <is>
+          <t>Вопрос</t>
+        </is>
+      </c>
+      <c r="D25" s="37" t="inlineStr">
+        <is>
+          <t>Ответ / комментарий</t>
+        </is>
+      </c>
+      <c r="E25" s="48" t="n"/>
+      <c r="F25" s="48" t="n"/>
+      <c r="G25" s="48" t="n"/>
+      <c r="H25" s="48" t="n"/>
+      <c r="I25" s="49" t="n"/>
+    </row>
+    <row r="26" ht="25.5" customHeight="1" s="47">
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>Что повлияло на трафик за неделю?</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E26" s="48" t="n"/>
+      <c r="F26" s="48" t="n"/>
+      <c r="G26" s="48" t="n"/>
+      <c r="H26" s="48" t="n"/>
+      <c r="I26" s="49" t="n"/>
+    </row>
+    <row r="27" ht="25.5" customHeight="1" s="47">
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Проблемы с оборудованием/химией</t>
+        </is>
+      </c>
+      <c r="D27" s="35" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E27" s="48" t="n"/>
+      <c r="F27" s="48" t="n"/>
+      <c r="G27" s="48" t="n"/>
+      <c r="H27" s="48" t="n"/>
+      <c r="I27" s="49" t="n"/>
+    </row>
+    <row r="28" ht="25.5" customHeight="1" s="47">
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Задачи на следующую неделю</t>
+        </is>
+      </c>
+      <c r="D28" s="35" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E28" s="48" t="n"/>
+      <c r="F28" s="48" t="n"/>
+      <c r="G28" s="48" t="n"/>
+      <c r="H28" s="48" t="n"/>
+      <c r="I28" s="49" t="n"/>
+    </row>
+    <row r="29" ht="25.5" customHeight="1" s="47">
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Что требует решения ГД?</t>
+        </is>
+      </c>
+      <c r="D29" s="35" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E29" s="48" t="n"/>
+      <c r="F29" s="48" t="n"/>
+      <c r="G29" s="48" t="n"/>
+      <c r="H29" s="48" t="n"/>
+      <c r="I29" s="49" t="n"/>
+    </row>
+    <row r="30" ht="7.5" customHeight="1" s="47"/>
+    <row r="31" ht="15.75" customHeight="1" s="47">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>🤖 Данные 1С — авто | 🖊 Комментарии — руководитель до 11:00 пн | Битрикс24</t>
+        </is>
+      </c>
+      <c r="B31" s="48" t="n"/>
+      <c r="C31" s="48" t="n"/>
+      <c r="D31" s="48" t="n"/>
+      <c r="E31" s="48" t="n"/>
+      <c r="F31" s="48" t="n"/>
+      <c r="G31" s="48" t="n"/>
+      <c r="H31" s="48" t="n"/>
+      <c r="I31" s="48" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D28:I28"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="D4:I4"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="D25:I25"/>
+    <mergeCell ref="D26:I26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2415,8 +2899,8 @@
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="D34:I34"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D38:I38"/>
     <mergeCell ref="A33:I33"/>
-    <mergeCell ref="D38:I38"/>
     <mergeCell ref="A42:I42"/>
     <mergeCell ref="D4:I4"/>
     <mergeCell ref="D5:I5"/>
@@ -3542,8 +4026,8 @@
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="D34:I34"/>
     <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D38:I38"/>
     <mergeCell ref="A33:I33"/>
-    <mergeCell ref="D38:I38"/>
     <mergeCell ref="A42:I42"/>
     <mergeCell ref="D4:I4"/>
     <mergeCell ref="D5:I5"/>

</xml_diff>

<commit_message>
Apply report template corrections
</commit_message>
<xml_diff>
--- a/backend/templates/report_template.xlsx
+++ b/backend/templates/report_template.xlsx
@@ -3,33 +3,34 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="713" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="713" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Арсенал (Д)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Арсенал (Н)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Реф.сервис (Д)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Реф.сервис (Н)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Шаркер (Д)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Шаркер (Н)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ЦКР (Д)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ЦКР (Н)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Мойка (Д)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Мойка ул. Строителей (Н)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Мойка Ульяновская (Н)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="СПРАВОЧНИК РУКОВОДИТЕЛЕЙ" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="Арсенал (Д)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Арсенал (Н)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Реф.сервис (Д)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Реф.сервис (Н)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Шаркер (Д)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Шаркер (Н)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ЦКР (Д)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ЦКР (Н)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Мойка (Д)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Мойка ул. Строителей (Н)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Мойка Ульяновская (Н)" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Арсенал (Д)'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Арсенал (Н)'!$A$1:$I$42</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Реф.сервис (Д)'!$A$1:$I$26</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Реф.сервис (Н)'!$A$1:$I$42</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Шаркер (Д)'!$A$1:$I$27</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Шаркер (Н)'!$A$1:$I$41</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="6">'ЦКР (Д)'!$A$1:$I$28</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="7">'ЦКР (Н)'!$A$1:$I$39</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Мойка (Д)'!$A$1:$I$17</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="9">'Мойка ул. Строителей (Н)'!$A$1:$I$31</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'Мойка Ульяновская (Н)'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Арсенал (Д)'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Арсенал (Н)'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Реф.сервис (Д)'!$A$1:$I$26</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Реф.сервис (Н)'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Шаркер (Д)'!$A$1:$I$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Шаркер (Н)'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'ЦКР (Д)'!$A$1:$I$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'ЦКР (Н)'!$A$1:$I$39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="9">'Мойка (Д)'!$A$1:$I$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'Мойка ул. Строителей (Н)'!$A$1:$I$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'Мойка Ульяновская (Н)'!$A$1:$I$31</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" refMode="R1C1"/>
 </workbook>
@@ -41,7 +42,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -201,8 +202,12 @@
       <color rgb="001F2933"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="22">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -325,8 +330,18 @@
         <fgColor rgb="005B9BD5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="31">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -664,11 +679,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <right/>
+      <bottom style="thin">
+        <color rgb="00B7C9D6"/>
+      </bottom>
+    </border>
+    <border>
+      <right/>
+      <bottom style="medium">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9DEE3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9DEE3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9DEE3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9DEE3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -891,6 +932,33 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="25" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="22" fillId="23" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -1148,9 +1216,111 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="47" min="1" max="1"/>
+    <col width="24" customWidth="1" style="47" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="88" t="inlineStr">
+        <is>
+          <t>Подразделение</t>
+        </is>
+      </c>
+      <c r="B1" s="88" t="inlineStr">
+        <is>
+          <t>ФИО</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="89" t="inlineStr">
+        <is>
+          <t>Арсенал</t>
+        </is>
+      </c>
+      <c r="B2" s="89" t="inlineStr">
+        <is>
+          <t>Мигунов А.А.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="89" t="inlineStr">
+        <is>
+          <t>Рефика Сервис</t>
+        </is>
+      </c>
+      <c r="B3" s="89" t="inlineStr">
+        <is>
+          <t>Михеев А.Н.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="89" t="inlineStr">
+        <is>
+          <t>Шаркер</t>
+        </is>
+      </c>
+      <c r="B4" s="89" t="inlineStr">
+        <is>
+          <t>Михеев А.Н.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="89" t="inlineStr">
+        <is>
+          <t>ЦКР</t>
+        </is>
+      </c>
+      <c r="B5" s="89" t="inlineStr">
+        <is>
+          <t>Игонин А.П.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="89" t="inlineStr">
+        <is>
+          <t>Мойка ул. Строителей</t>
+        </is>
+      </c>
+      <c r="B6" s="89" t="inlineStr">
+        <is>
+          <t>Расторгуев С.В.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="89" t="inlineStr">
+        <is>
+          <t>Мойка ул. Ульяновская</t>
+        </is>
+      </c>
+      <c r="B7" s="89" t="inlineStr">
+        <is>
+          <t>Расторгуев С.В.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="47" min="1" max="1"/>
@@ -1167,9 +1337,9 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
-        <is>
-          <t>ЕЖЕДНЕВНЫЙ ОТЧЁТ — АРСЕНАЛ  |  Данные из 1С</t>
+      <c r="A1" s="90" t="inlineStr">
+        <is>
+          <t>ЕЖЕДНЕВНЫЙ ОТЧЁТ — МОЙКА  |  Данные из 1С</t>
         </is>
       </c>
       <c r="B1" s="75" t="n"/>
@@ -1181,8 +1351,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -1240,7 +1410,7 @@
     <row r="6" ht="33" customHeight="1" s="47">
       <c r="A6" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ВЫРАБОТКА</t>
+          <t xml:space="preserve">  КЛЮЧЕВЫЕ ПОКАЗАТЕЛИ (из 1С) Мойка на ул. Строителей</t>
         </is>
       </c>
       <c r="B6" s="79" t="n"/>
@@ -1287,7 +1457,7 @@
       <c r="A8" s="69" t="n"/>
       <c r="B8" s="69" t="inlineStr">
         <is>
-          <t>Нормочасы за день — общая выработка</t>
+          <t>Машин обслужено</t>
         </is>
       </c>
       <c r="C8" s="70" t="n"/>
@@ -1301,7 +1471,7 @@
       </c>
       <c r="I8" s="70" t="inlineStr">
         <is>
-          <t>нч</t>
+          <t>шт.</t>
         </is>
       </c>
     </row>
@@ -1309,7 +1479,7 @@
       <c r="A9" s="69" t="n"/>
       <c r="B9" s="69" t="inlineStr">
         <is>
-          <t>Выработка на 1 мастера (нч/чел.)</t>
+          <t>Выручка за день</t>
         </is>
       </c>
       <c r="C9" s="70" t="n"/>
@@ -1323,7 +1493,7 @@
       </c>
       <c r="I9" s="70" t="inlineStr">
         <is>
-          <t>нч/чел</t>
+          <t>руб.</t>
         </is>
       </c>
     </row>
@@ -1331,13 +1501,19 @@
       <c r="A10" s="69" t="n"/>
       <c r="B10" s="69" t="inlineStr">
         <is>
-          <t>Закрыто ЗН за день</t>
+          <t>Средний чек (руб./машина)</t>
         </is>
       </c>
       <c r="C10" s="70" t="n"/>
-      <c r="D10" s="81" t="n"/>
+      <c r="D10" s="81">
+        <f>IFERROR(D9/D8,"—")</f>
+        <v/>
+      </c>
       <c r="E10" s="70" t="n"/>
-      <c r="F10" s="81" t="n"/>
+      <c r="F10" s="81">
+        <f>IFERROR(F9/F8,"—")</f>
+        <v/>
+      </c>
       <c r="G10" s="70" t="n"/>
       <c r="H10" s="82">
         <f>IFERROR(IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&gt;0),F10/D10,"—"),"—")</f>
@@ -1345,7 +1521,7 @@
       </c>
       <c r="I10" s="70" t="inlineStr">
         <is>
-          <t>шт.</t>
+          <t>руб.</t>
         </is>
       </c>
     </row>
@@ -1360,19 +1536,19 @@
       <c r="H11" s="83" t="n"/>
       <c r="I11" s="55" t="n"/>
     </row>
-    <row r="12" ht="33" customHeight="1" s="47">
+    <row r="12" ht="33" customHeight="1" s="47" thickBot="1">
       <c r="A12" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ФИНАНСЫ</t>
+          <t xml:space="preserve">  КЛЮЧЕВЫЕ ПОКАЗАТЕЛИ (из 1С) Мойка на ул. Ульяновская</t>
         </is>
       </c>
       <c r="B12" s="79" t="n"/>
       <c r="C12" s="79" t="n"/>
-      <c r="D12" s="84" t="n"/>
+      <c r="D12" s="79" t="n"/>
       <c r="E12" s="79" t="n"/>
-      <c r="F12" s="84" t="n"/>
+      <c r="F12" s="79" t="n"/>
       <c r="G12" s="79" t="n"/>
-      <c r="H12" s="84" t="n"/>
+      <c r="H12" s="79" t="n"/>
       <c r="I12" s="80" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1" s="47">
@@ -1410,7 +1586,7 @@
       <c r="A14" s="69" t="n"/>
       <c r="B14" s="69" t="inlineStr">
         <is>
-          <t>Выручка за день</t>
+          <t>Машин обслужено</t>
         </is>
       </c>
       <c r="C14" s="70" t="n"/>
@@ -1424,7 +1600,7 @@
       </c>
       <c r="I14" s="70" t="inlineStr">
         <is>
-          <t>руб.</t>
+          <t>шт.</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1608,7 @@
       <c r="A15" s="69" t="n"/>
       <c r="B15" s="69" t="inlineStr">
         <is>
-          <t>Себестоимость ЗЧ</t>
+          <t>Выручка за день</t>
         </is>
       </c>
       <c r="C15" s="70" t="n"/>
@@ -1454,17 +1630,17 @@
       <c r="A16" s="69" t="n"/>
       <c r="B16" s="69" t="inlineStr">
         <is>
-          <t>Маржа (Выручка − Себест. ЗЧ)</t>
+          <t>Средний чек (руб./машина)</t>
         </is>
       </c>
       <c r="C16" s="70" t="n"/>
       <c r="D16" s="81">
-        <f>IFERROR(D14-D15,"—")</f>
+        <f>IFERROR(D15/D14,"—")</f>
         <v/>
       </c>
       <c r="E16" s="70" t="n"/>
       <c r="F16" s="81">
-        <f>IFERROR(F14-F15,"—")</f>
+        <f>IFERROR(F15/F14,"—")</f>
         <v/>
       </c>
       <c r="G16" s="70" t="n"/>
@@ -1479,814 +1655,29 @@
       </c>
     </row>
     <row r="17" ht="33" customHeight="1" s="47">
-      <c r="A17" s="69" t="n"/>
-      <c r="B17" s="69" t="inlineStr">
-        <is>
-          <t>Маржинальность</t>
-        </is>
-      </c>
-      <c r="C17" s="70" t="n"/>
-      <c r="D17" s="82">
-        <f>IFERROR(D16/D14,"—")</f>
-        <v/>
-      </c>
-      <c r="E17" s="70" t="n"/>
-      <c r="F17" s="82">
-        <f>IFERROR(F16/F14,"—")</f>
-        <v/>
-      </c>
-      <c r="G17" s="70" t="n"/>
-      <c r="H17" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D17),ISNUMBER(F17),D17&gt;0),F17/D17,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I17" s="70" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="33" customHeight="1" s="47">
-      <c r="A18" s="69" t="n"/>
-      <c r="B18" s="69" t="inlineStr">
-        <is>
-          <t>Средний чек (руб./ЗН)</t>
-        </is>
-      </c>
-      <c r="C18" s="70" t="n"/>
-      <c r="D18" s="81">
-        <f>IFERROR(D14/D10,"—")</f>
-        <v/>
-      </c>
-      <c r="E18" s="70" t="n"/>
-      <c r="F18" s="81">
-        <f>IFERROR(F14/F10,"—")</f>
-        <v/>
-      </c>
-      <c r="G18" s="70" t="n"/>
-      <c r="H18" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D18),ISNUMBER(F18),D18&gt;0),F18/D18,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I18" s="70" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="33" customHeight="1" s="47">
-      <c r="A19" s="69" t="n"/>
-      <c r="B19" s="69" t="inlineStr">
-        <is>
-          <t>Наценка на ЗЧ</t>
-        </is>
-      </c>
-      <c r="C19" s="70" t="n"/>
-      <c r="D19" s="82" t="n"/>
-      <c r="E19" s="70" t="n"/>
-      <c r="F19" s="82" t="n"/>
-      <c r="G19" s="70" t="n"/>
-      <c r="H19" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D19),ISNUMBER(F19),D19&gt;0),F19/D19,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I19" s="70" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="8" customHeight="1" s="47">
-      <c r="A20" s="55" t="n"/>
-      <c r="B20" s="55" t="n"/>
-      <c r="C20" s="55" t="n"/>
-      <c r="D20" s="83" t="n"/>
-      <c r="E20" s="55" t="n"/>
-      <c r="F20" s="83" t="n"/>
-      <c r="G20" s="55" t="n"/>
-      <c r="H20" s="83" t="n"/>
-      <c r="I20" s="55" t="n"/>
-    </row>
-    <row r="21" ht="33" customHeight="1" s="47">
-      <c r="A21" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  СНАБЖЕНИЕ (из 1С)</t>
-        </is>
-      </c>
-      <c r="B21" s="79" t="n"/>
-      <c r="C21" s="79" t="n"/>
-      <c r="D21" s="84" t="n"/>
-      <c r="E21" s="79" t="n"/>
-      <c r="F21" s="84" t="n"/>
-      <c r="G21" s="79" t="n"/>
-      <c r="H21" s="84" t="n"/>
-      <c r="I21" s="80" t="n"/>
-    </row>
-    <row r="22" ht="33" customHeight="1" s="47">
-      <c r="A22" s="68" t="n"/>
-      <c r="B22" s="68" t="inlineStr">
-        <is>
-          <t>Показатель</t>
-        </is>
-      </c>
-      <c r="C22" s="68" t="n"/>
-      <c r="D22" s="68" t="inlineStr">
-        <is>
-          <t>Значение (1С)</t>
-        </is>
-      </c>
-      <c r="E22" s="77" t="n"/>
-      <c r="F22" s="85" t="n"/>
-      <c r="G22" s="68" t="n"/>
-      <c r="H22" s="68" t="inlineStr">
-        <is>
-          <t>Норма</t>
-        </is>
-      </c>
-      <c r="I22" s="78" t="n"/>
-    </row>
-    <row r="23" ht="33" customHeight="1" s="47">
-      <c r="A23" s="69" t="n"/>
-      <c r="B23" s="69" t="inlineStr">
-        <is>
-          <t>Незакрытые ЗН старше 1 дня (шт.)</t>
-        </is>
-      </c>
-      <c r="C23" s="70" t="n"/>
-      <c r="D23" s="81" t="n"/>
-      <c r="E23" s="77" t="n"/>
-      <c r="F23" s="85" t="n"/>
-      <c r="G23" s="70" t="n"/>
-      <c r="H23" s="70" t="inlineStr">
-        <is>
-          <t>Цель: 0</t>
-        </is>
-      </c>
-      <c r="I23" s="78" t="n"/>
-    </row>
-    <row r="24" ht="33" customHeight="1" s="47">
-      <c r="A24" s="69" t="n"/>
-      <c r="B24" s="69" t="inlineStr">
-        <is>
-          <t>ЗН без движения &gt; 2 дней (шт.)</t>
-        </is>
-      </c>
-      <c r="C24" s="70" t="n"/>
-      <c r="D24" s="81" t="n"/>
-      <c r="E24" s="77" t="n"/>
-      <c r="F24" s="85" t="n"/>
-      <c r="G24" s="70" t="n"/>
-      <c r="H24" s="70" t="inlineStr">
-        <is>
-          <t>Цель: 0</t>
-        </is>
-      </c>
-      <c r="I24" s="78" t="n"/>
-    </row>
-    <row r="25" ht="8" customHeight="1" s="47">
-      <c r="A25" s="55" t="n"/>
-      <c r="B25" s="55" t="n"/>
-      <c r="C25" s="55" t="n"/>
-      <c r="D25" s="83" t="n"/>
-      <c r="E25" s="55" t="n"/>
-      <c r="F25" s="83" t="n"/>
-      <c r="G25" s="55" t="n"/>
-      <c r="H25" s="83" t="n"/>
-      <c r="I25" s="55" t="n"/>
-    </row>
-    <row r="26" ht="33" customHeight="1" s="47">
-      <c r="A26" s="69" t="inlineStr">
+      <c r="A17" s="69" t="inlineStr">
         <is>
           <t>🤖 Генерируется автоматически в 11:00 | Данные: 1С Альфа-Авто | Отправка: Битрикс24</t>
         </is>
       </c>
-      <c r="B26" s="77" t="n"/>
-      <c r="C26" s="77" t="n"/>
-      <c r="D26" s="86" t="n"/>
-      <c r="E26" s="77" t="n"/>
-      <c r="F26" s="86" t="n"/>
-      <c r="G26" s="77" t="n"/>
-      <c r="H26" s="86" t="n"/>
-      <c r="I26" s="78" t="n"/>
+      <c r="B17" s="77" t="n"/>
+      <c r="C17" s="77" t="n"/>
+      <c r="D17" s="77" t="n"/>
+      <c r="E17" s="77" t="n"/>
+      <c r="F17" s="77" t="n"/>
+      <c r="G17" s="77" t="n"/>
+      <c r="H17" s="77" t="n"/>
+      <c r="I17" s="78" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="7">
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="D23:F23"/>
     <mergeCell ref="D4:I4"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="D22:F22"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="A17:I17"/>
+    <mergeCell ref="A6:I6"/>
     <mergeCell ref="D3:I3"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="H22:I22"/>
     <mergeCell ref="A12:I12"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A21:I21"/>
-    <mergeCell ref="D24:F24"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:I31"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" style="47" min="1" max="1"/>
-    <col width="48" customWidth="1" style="47" min="2" max="2"/>
-    <col width="2" customWidth="1" style="47" min="3" max="3"/>
-    <col width="15" customWidth="1" style="47" min="4" max="4"/>
-    <col width="2" customWidth="1" style="47" min="5" max="5"/>
-    <col width="15" customWidth="1" style="47" min="6" max="6"/>
-    <col width="2" customWidth="1" style="47" min="7" max="7"/>
-    <col width="14" customWidth="1" style="47" min="8" max="8"/>
-    <col width="16" customWidth="1" style="47" min="9" max="9"/>
-    <col hidden="1" width="2" customWidth="1" style="47" min="10" max="10"/>
-    <col hidden="1" width="2" customWidth="1" style="47" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
-        <is>
-          <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — МОЙКА</t>
-        </is>
-      </c>
-      <c r="B1" s="75" t="n"/>
-      <c r="C1" s="75" t="n"/>
-      <c r="D1" s="75" t="n"/>
-      <c r="E1" s="75" t="n"/>
-      <c r="F1" s="75" t="n"/>
-      <c r="G1" s="75" t="n"/>
-      <c r="H1" s="75" t="n"/>
-      <c r="I1" s="75" t="n"/>
-    </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
-        </is>
-      </c>
-      <c r="B2" s="76" t="n"/>
-      <c r="C2" s="76" t="n"/>
-      <c r="D2" s="76" t="n"/>
-      <c r="E2" s="76" t="n"/>
-      <c r="F2" s="76" t="n"/>
-      <c r="G2" s="76" t="n"/>
-      <c r="H2" s="76" t="n"/>
-      <c r="I2" s="76" t="n"/>
-    </row>
-    <row r="3" ht="30" customHeight="1" s="47">
-      <c r="A3" s="64" t="n"/>
-      <c r="B3" s="65" t="inlineStr">
-        <is>
-          <t>АТЦ:</t>
-        </is>
-      </c>
-      <c r="C3" s="64" t="n"/>
-      <c r="D3" s="66" t="n"/>
-      <c r="E3" s="77" t="n"/>
-      <c r="F3" s="77" t="n"/>
-      <c r="G3" s="77" t="n"/>
-      <c r="H3" s="77" t="n"/>
-      <c r="I3" s="78" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1" s="47">
-      <c r="A4" s="64" t="n"/>
-      <c r="B4" s="65" t="inlineStr">
-        <is>
-          <t>Неделя (авто):</t>
-        </is>
-      </c>
-      <c r="C4" s="64" t="n"/>
-      <c r="D4" s="66" t="n"/>
-      <c r="E4" s="77" t="n"/>
-      <c r="F4" s="77" t="n"/>
-      <c r="G4" s="77" t="n"/>
-      <c r="H4" s="77" t="n"/>
-      <c r="I4" s="78" t="n"/>
-    </row>
-    <row r="5" ht="30" customHeight="1" s="47">
-      <c r="A5" s="64" t="n"/>
-      <c r="B5" s="65" t="inlineStr">
-        <is>
-          <t>Руководитель (авто):</t>
-        </is>
-      </c>
-      <c r="C5" s="64" t="n"/>
-      <c r="D5" s="66" t="n"/>
-      <c r="E5" s="77" t="n"/>
-      <c r="F5" s="77" t="n"/>
-      <c r="G5" s="77" t="n"/>
-      <c r="H5" s="77" t="n"/>
-      <c r="I5" s="78" t="n"/>
-    </row>
-    <row r="6" ht="8" customHeight="1" s="47">
-      <c r="A6" s="55" t="n"/>
-      <c r="B6" s="55" t="n"/>
-      <c r="C6" s="55" t="n"/>
-      <c r="D6" s="55" t="n"/>
-      <c r="E6" s="55" t="n"/>
-      <c r="F6" s="55" t="n"/>
-      <c r="G6" s="55" t="n"/>
-      <c r="H6" s="55" t="n"/>
-      <c r="I6" s="55" t="n"/>
-    </row>
-    <row r="7" ht="33" customHeight="1" s="47">
-      <c r="A7" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1.  КЛЮЧЕВЫЕ ПОКАЗАТЕЛИ  [из 1С]</t>
-        </is>
-      </c>
-      <c r="B7" s="79" t="n"/>
-      <c r="C7" s="79" t="n"/>
-      <c r="D7" s="79" t="n"/>
-      <c r="E7" s="79" t="n"/>
-      <c r="F7" s="79" t="n"/>
-      <c r="G7" s="79" t="n"/>
-      <c r="H7" s="79" t="n"/>
-      <c r="I7" s="80" t="n"/>
-    </row>
-    <row r="8" ht="33" customHeight="1" s="47">
-      <c r="A8" s="68" t="n"/>
-      <c r="B8" s="68" t="inlineStr">
-        <is>
-          <t>Показатель</t>
-        </is>
-      </c>
-      <c r="C8" s="68" t="n"/>
-      <c r="D8" s="68" t="inlineStr">
-        <is>
-          <t>ПЛАН</t>
-        </is>
-      </c>
-      <c r="E8" s="68" t="n"/>
-      <c r="F8" s="68" t="inlineStr">
-        <is>
-          <t>ФАКТ (1С)</t>
-        </is>
-      </c>
-      <c r="G8" s="68" t="n"/>
-      <c r="H8" s="68" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="I8" s="68" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="33" customHeight="1" s="47">
-      <c r="A9" s="69" t="n"/>
-      <c r="B9" s="69" t="inlineStr">
-        <is>
-          <t>Машин за неделю</t>
-        </is>
-      </c>
-      <c r="C9" s="70" t="n"/>
-      <c r="D9" s="81" t="n"/>
-      <c r="E9" s="70" t="n"/>
-      <c r="F9" s="81" t="n"/>
-      <c r="G9" s="70" t="n"/>
-      <c r="H9" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9&gt;0),F9/D9,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I9" s="70" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="33" customHeight="1" s="47">
-      <c r="A10" s="69" t="n"/>
-      <c r="B10" s="69" t="inlineStr">
-        <is>
-          <t>Выручка за неделю</t>
-        </is>
-      </c>
-      <c r="C10" s="70" t="n"/>
-      <c r="D10" s="81" t="n"/>
-      <c r="E10" s="70" t="n"/>
-      <c r="F10" s="81" t="n"/>
-      <c r="G10" s="70" t="n"/>
-      <c r="H10" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&gt;0),F10/D10,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I10" s="70" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="33" customHeight="1" s="47">
-      <c r="A11" s="69" t="n"/>
-      <c r="B11" s="69" t="inlineStr">
-        <is>
-          <t>Средний чек</t>
-        </is>
-      </c>
-      <c r="C11" s="70" t="n"/>
-      <c r="D11" s="81">
-        <f>IFERROR(D10/D9,"—")</f>
-        <v/>
-      </c>
-      <c r="E11" s="70" t="n"/>
-      <c r="F11" s="81">
-        <f>IFERROR(F10/F9,"—")</f>
-        <v/>
-      </c>
-      <c r="G11" s="70" t="n"/>
-      <c r="H11" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D11),ISNUMBER(F11),D11&gt;0),F11/D11,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I11" s="70" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="8" customHeight="1" s="47">
-      <c r="A12" s="55" t="n"/>
-      <c r="B12" s="55" t="n"/>
-      <c r="C12" s="55" t="n"/>
-      <c r="D12" s="83" t="n"/>
-      <c r="E12" s="55" t="n"/>
-      <c r="F12" s="83" t="n"/>
-      <c r="G12" s="55" t="n"/>
-      <c r="H12" s="83" t="n"/>
-      <c r="I12" s="55" t="n"/>
-    </row>
-    <row r="13" ht="33" customHeight="1" s="47">
-      <c r="A13" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2.  ДИНАМИКА ПО ДНЯМ  [из 1С]</t>
-        </is>
-      </c>
-      <c r="B13" s="79" t="n"/>
-      <c r="C13" s="79" t="n"/>
-      <c r="D13" s="84" t="n"/>
-      <c r="E13" s="79" t="n"/>
-      <c r="F13" s="84" t="n"/>
-      <c r="G13" s="79" t="n"/>
-      <c r="H13" s="84" t="n"/>
-      <c r="I13" s="80" t="n"/>
-    </row>
-    <row r="14" ht="33" customHeight="1" s="47">
-      <c r="A14" s="69" t="n"/>
-      <c r="B14" s="69" t="inlineStr">
-        <is>
-          <t>День</t>
-        </is>
-      </c>
-      <c r="C14" s="70" t="n"/>
-      <c r="D14" s="70" t="inlineStr">
-        <is>
-          <t>Машин</t>
-        </is>
-      </c>
-      <c r="E14" s="70" t="n"/>
-      <c r="F14" s="70" t="inlineStr">
-        <is>
-          <t>Выручка</t>
-        </is>
-      </c>
-      <c r="G14" s="70" t="n"/>
-      <c r="H14" s="70" t="inlineStr">
-        <is>
-          <t>Ср.чек</t>
-        </is>
-      </c>
-      <c r="I14" s="70" t="inlineStr">
-        <is>
-          <t>Операторов</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="33" customHeight="1" s="47">
-      <c r="A15" s="69" t="n"/>
-      <c r="B15" s="69" t="inlineStr">
-        <is>
-          <t>Пн</t>
-        </is>
-      </c>
-      <c r="C15" s="70" t="n"/>
-      <c r="D15" s="81" t="n"/>
-      <c r="E15" s="70" t="n"/>
-      <c r="F15" s="81" t="n"/>
-      <c r="G15" s="70" t="n"/>
-      <c r="H15" s="81">
-        <f>IFERROR(F15/D15,"—")</f>
-        <v/>
-      </c>
-      <c r="I15" s="70" t="n"/>
-    </row>
-    <row r="16" ht="33" customHeight="1" s="47">
-      <c r="A16" s="69" t="n"/>
-      <c r="B16" s="69" t="inlineStr">
-        <is>
-          <t>Вт</t>
-        </is>
-      </c>
-      <c r="C16" s="70" t="n"/>
-      <c r="D16" s="81" t="n"/>
-      <c r="E16" s="70" t="n"/>
-      <c r="F16" s="81" t="n"/>
-      <c r="G16" s="70" t="n"/>
-      <c r="H16" s="81">
-        <f>IFERROR(F16/D16,"—")</f>
-        <v/>
-      </c>
-      <c r="I16" s="70" t="n"/>
-    </row>
-    <row r="17" ht="33" customHeight="1" s="47">
-      <c r="A17" s="69" t="n"/>
-      <c r="B17" s="69" t="inlineStr">
-        <is>
-          <t>Ср</t>
-        </is>
-      </c>
-      <c r="C17" s="70" t="n"/>
-      <c r="D17" s="81" t="n"/>
-      <c r="E17" s="70" t="n"/>
-      <c r="F17" s="81" t="n"/>
-      <c r="G17" s="70" t="n"/>
-      <c r="H17" s="81">
-        <f>IFERROR(F17/D17,"—")</f>
-        <v/>
-      </c>
-      <c r="I17" s="70" t="n"/>
-    </row>
-    <row r="18" ht="33" customHeight="1" s="47">
-      <c r="A18" s="69" t="n"/>
-      <c r="B18" s="69" t="inlineStr">
-        <is>
-          <t>Чт</t>
-        </is>
-      </c>
-      <c r="C18" s="70" t="n"/>
-      <c r="D18" s="81" t="n"/>
-      <c r="E18" s="70" t="n"/>
-      <c r="F18" s="81" t="n"/>
-      <c r="G18" s="70" t="n"/>
-      <c r="H18" s="81">
-        <f>IFERROR(F18/D18,"—")</f>
-        <v/>
-      </c>
-      <c r="I18" s="70" t="n"/>
-    </row>
-    <row r="19" ht="33" customHeight="1" s="47">
-      <c r="A19" s="69" t="n"/>
-      <c r="B19" s="69" t="inlineStr">
-        <is>
-          <t>Пт</t>
-        </is>
-      </c>
-      <c r="C19" s="70" t="n"/>
-      <c r="D19" s="81" t="n"/>
-      <c r="E19" s="70" t="n"/>
-      <c r="F19" s="81" t="n"/>
-      <c r="G19" s="70" t="n"/>
-      <c r="H19" s="81">
-        <f>IFERROR(F19/D19,"—")</f>
-        <v/>
-      </c>
-      <c r="I19" s="70" t="n"/>
-    </row>
-    <row r="20" ht="33" customHeight="1" s="47">
-      <c r="A20" s="69" t="n"/>
-      <c r="B20" s="69" t="inlineStr">
-        <is>
-          <t>Сб</t>
-        </is>
-      </c>
-      <c r="C20" s="70" t="n"/>
-      <c r="D20" s="81" t="n"/>
-      <c r="E20" s="70" t="n"/>
-      <c r="F20" s="81" t="n"/>
-      <c r="G20" s="70" t="n"/>
-      <c r="H20" s="81">
-        <f>IFERROR(F20/D20,"—")</f>
-        <v/>
-      </c>
-      <c r="I20" s="70" t="n"/>
-    </row>
-    <row r="21" ht="33" customHeight="1" s="47">
-      <c r="A21" s="69" t="n"/>
-      <c r="B21" s="69" t="inlineStr">
-        <is>
-          <t>Вс</t>
-        </is>
-      </c>
-      <c r="C21" s="70" t="n"/>
-      <c r="D21" s="81" t="n"/>
-      <c r="E21" s="70" t="n"/>
-      <c r="F21" s="81" t="n"/>
-      <c r="G21" s="70" t="n"/>
-      <c r="H21" s="81">
-        <f>IFERROR(F21/D21,"—")</f>
-        <v/>
-      </c>
-      <c r="I21" s="70" t="n"/>
-    </row>
-    <row r="22" ht="33" customHeight="1" s="47">
-      <c r="A22" s="69" t="n"/>
-      <c r="B22" s="69" t="inlineStr">
-        <is>
-          <t>ИТОГО</t>
-        </is>
-      </c>
-      <c r="C22" s="70" t="n"/>
-      <c r="D22" s="81">
-        <f>SUM(D15:D21)</f>
-        <v/>
-      </c>
-      <c r="E22" s="70" t="n"/>
-      <c r="F22" s="81">
-        <f>SUM(F15:F21)</f>
-        <v/>
-      </c>
-      <c r="G22" s="70" t="n"/>
-      <c r="H22" s="81">
-        <f>IFERROR(F22/D22,"—")</f>
-        <v/>
-      </c>
-      <c r="I22" s="70" t="n"/>
-    </row>
-    <row r="23" ht="8" customHeight="1" s="47">
-      <c r="A23" s="55" t="n"/>
-      <c r="B23" s="55" t="n"/>
-      <c r="C23" s="55" t="n"/>
-      <c r="D23" s="83" t="n"/>
-      <c r="E23" s="55" t="n"/>
-      <c r="F23" s="83" t="n"/>
-      <c r="G23" s="55" t="n"/>
-      <c r="H23" s="83" t="n"/>
-      <c r="I23" s="55" t="n"/>
-    </row>
-    <row r="24" ht="33" customHeight="1" s="47">
-      <c r="A24" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  3.  КОММЕНТАРИЙ РУКОВОДИТЕЛЯ  [вручную]</t>
-        </is>
-      </c>
-      <c r="B24" s="79" t="n"/>
-      <c r="C24" s="79" t="n"/>
-      <c r="D24" s="84" t="n"/>
-      <c r="E24" s="79" t="n"/>
-      <c r="F24" s="84" t="n"/>
-      <c r="G24" s="79" t="n"/>
-      <c r="H24" s="84" t="n"/>
-      <c r="I24" s="80" t="n"/>
-    </row>
-    <row r="25" ht="33" customHeight="1" s="47">
-      <c r="A25" s="69" t="n"/>
-      <c r="B25" s="69" t="inlineStr">
-        <is>
-          <t>Вопрос</t>
-        </is>
-      </c>
-      <c r="C25" s="70" t="n"/>
-      <c r="D25" s="70" t="inlineStr">
-        <is>
-          <t>Ответ / комментарий</t>
-        </is>
-      </c>
-      <c r="E25" s="77" t="n"/>
-      <c r="F25" s="86" t="n"/>
-      <c r="G25" s="77" t="n"/>
-      <c r="H25" s="86" t="n"/>
-      <c r="I25" s="78" t="n"/>
-    </row>
-    <row r="26" ht="33" customHeight="1" s="47">
-      <c r="A26" s="69" t="n"/>
-      <c r="B26" s="69" t="inlineStr">
-        <is>
-          <t>Что повлияло на трафик за неделю?</t>
-        </is>
-      </c>
-      <c r="C26" s="70" t="n"/>
-      <c r="D26" s="70" t="inlineStr">
-        <is>
-          <t>введите комментарий...</t>
-        </is>
-      </c>
-      <c r="E26" s="77" t="n"/>
-      <c r="F26" s="86" t="n"/>
-      <c r="G26" s="77" t="n"/>
-      <c r="H26" s="86" t="n"/>
-      <c r="I26" s="78" t="n"/>
-    </row>
-    <row r="27" ht="33" customHeight="1" s="47">
-      <c r="A27" s="69" t="n"/>
-      <c r="B27" s="69" t="inlineStr">
-        <is>
-          <t>Проблемы с оборудованием/химией</t>
-        </is>
-      </c>
-      <c r="C27" s="70" t="n"/>
-      <c r="D27" s="70" t="inlineStr">
-        <is>
-          <t>введите комментарий...</t>
-        </is>
-      </c>
-      <c r="E27" s="77" t="n"/>
-      <c r="F27" s="86" t="n"/>
-      <c r="G27" s="77" t="n"/>
-      <c r="H27" s="86" t="n"/>
-      <c r="I27" s="78" t="n"/>
-    </row>
-    <row r="28" ht="33" customHeight="1" s="47">
-      <c r="A28" s="69" t="n"/>
-      <c r="B28" s="69" t="inlineStr">
-        <is>
-          <t>Задачи на следующую неделю</t>
-        </is>
-      </c>
-      <c r="C28" s="70" t="n"/>
-      <c r="D28" s="70" t="inlineStr">
-        <is>
-          <t>введите комментарий...</t>
-        </is>
-      </c>
-      <c r="E28" s="77" t="n"/>
-      <c r="F28" s="86" t="n"/>
-      <c r="G28" s="77" t="n"/>
-      <c r="H28" s="86" t="n"/>
-      <c r="I28" s="78" t="n"/>
-    </row>
-    <row r="29" ht="33" customHeight="1" s="47">
-      <c r="A29" s="69" t="n"/>
-      <c r="B29" s="69" t="inlineStr">
-        <is>
-          <t>Что требует решения ГД?</t>
-        </is>
-      </c>
-      <c r="C29" s="70" t="n"/>
-      <c r="D29" s="70" t="inlineStr">
-        <is>
-          <t>введите комментарий...</t>
-        </is>
-      </c>
-      <c r="E29" s="77" t="n"/>
-      <c r="F29" s="86" t="n"/>
-      <c r="G29" s="77" t="n"/>
-      <c r="H29" s="86" t="n"/>
-      <c r="I29" s="78" t="n"/>
-    </row>
-    <row r="30" ht="8" customHeight="1" s="47">
-      <c r="A30" s="55" t="n"/>
-      <c r="B30" s="55" t="n"/>
-      <c r="C30" s="55" t="n"/>
-      <c r="D30" s="83" t="n"/>
-      <c r="E30" s="55" t="n"/>
-      <c r="F30" s="83" t="n"/>
-      <c r="G30" s="55" t="n"/>
-      <c r="H30" s="83" t="n"/>
-      <c r="I30" s="55" t="n"/>
-    </row>
-    <row r="31" ht="33" customHeight="1" s="47">
-      <c r="A31" s="69" t="inlineStr">
-        <is>
-          <t>🤖 Данные 1С — авто | 🖊 Комментарии — руководитель до 11:00 пн | Битрикс24</t>
-        </is>
-      </c>
-      <c r="B31" s="77" t="n"/>
-      <c r="C31" s="77" t="n"/>
-      <c r="D31" s="86" t="n"/>
-      <c r="E31" s="77" t="n"/>
-      <c r="F31" s="86" t="n"/>
-      <c r="G31" s="77" t="n"/>
-      <c r="H31" s="86" t="n"/>
-      <c r="I31" s="78" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="A7:I7"/>
-    <mergeCell ref="D27:I27"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="D28:I28"/>
-    <mergeCell ref="D29:I29"/>
-    <mergeCell ref="D4:I4"/>
-    <mergeCell ref="D5:I5"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="D25:I25"/>
-    <mergeCell ref="D26:I26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
@@ -2316,7 +1707,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — МОЙКА</t>
         </is>
@@ -2330,8 +1721,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -2538,11 +1929,11 @@
       </c>
       <c r="B13" s="79" t="n"/>
       <c r="C13" s="79" t="n"/>
-      <c r="D13" s="84" t="n"/>
+      <c r="D13" s="79" t="n"/>
       <c r="E13" s="79" t="n"/>
-      <c r="F13" s="84" t="n"/>
+      <c r="F13" s="79" t="n"/>
       <c r="G13" s="79" t="n"/>
-      <c r="H13" s="84" t="n"/>
+      <c r="H13" s="79" t="n"/>
       <c r="I13" s="80" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
@@ -2745,11 +2136,11 @@
       </c>
       <c r="B24" s="79" t="n"/>
       <c r="C24" s="79" t="n"/>
-      <c r="D24" s="84" t="n"/>
+      <c r="D24" s="79" t="n"/>
       <c r="E24" s="79" t="n"/>
-      <c r="F24" s="84" t="n"/>
+      <c r="F24" s="79" t="n"/>
       <c r="G24" s="79" t="n"/>
-      <c r="H24" s="84" t="n"/>
+      <c r="H24" s="79" t="n"/>
       <c r="I24" s="80" t="n"/>
     </row>
     <row r="25" ht="33" customHeight="1" s="47">
@@ -2766,9 +2157,9 @@
         </is>
       </c>
       <c r="E25" s="77" t="n"/>
-      <c r="F25" s="86" t="n"/>
+      <c r="F25" s="77" t="n"/>
       <c r="G25" s="77" t="n"/>
-      <c r="H25" s="86" t="n"/>
+      <c r="H25" s="77" t="n"/>
       <c r="I25" s="78" t="n"/>
     </row>
     <row r="26" ht="33" customHeight="1" s="47">
@@ -2785,9 +2176,9 @@
         </is>
       </c>
       <c r="E26" s="77" t="n"/>
-      <c r="F26" s="86" t="n"/>
+      <c r="F26" s="77" t="n"/>
       <c r="G26" s="77" t="n"/>
-      <c r="H26" s="86" t="n"/>
+      <c r="H26" s="77" t="n"/>
       <c r="I26" s="78" t="n"/>
     </row>
     <row r="27" ht="33" customHeight="1" s="47">
@@ -2804,9 +2195,9 @@
         </is>
       </c>
       <c r="E27" s="77" t="n"/>
-      <c r="F27" s="86" t="n"/>
+      <c r="F27" s="77" t="n"/>
       <c r="G27" s="77" t="n"/>
-      <c r="H27" s="86" t="n"/>
+      <c r="H27" s="77" t="n"/>
       <c r="I27" s="78" t="n"/>
     </row>
     <row r="28" ht="33" customHeight="1" s="47">
@@ -2823,9 +2214,9 @@
         </is>
       </c>
       <c r="E28" s="77" t="n"/>
-      <c r="F28" s="86" t="n"/>
+      <c r="F28" s="77" t="n"/>
       <c r="G28" s="77" t="n"/>
-      <c r="H28" s="86" t="n"/>
+      <c r="H28" s="77" t="n"/>
       <c r="I28" s="78" t="n"/>
     </row>
     <row r="29" ht="33" customHeight="1" s="47">
@@ -2842,9 +2233,9 @@
         </is>
       </c>
       <c r="E29" s="77" t="n"/>
-      <c r="F29" s="86" t="n"/>
+      <c r="F29" s="77" t="n"/>
       <c r="G29" s="77" t="n"/>
-      <c r="H29" s="86" t="n"/>
+      <c r="H29" s="77" t="n"/>
       <c r="I29" s="78" t="n"/>
     </row>
     <row r="30" ht="8" customHeight="1" s="47">
@@ -2866,11 +2257,613 @@
       </c>
       <c r="B31" s="77" t="n"/>
       <c r="C31" s="77" t="n"/>
-      <c r="D31" s="86" t="n"/>
+      <c r="D31" s="77" t="n"/>
       <c r="E31" s="77" t="n"/>
-      <c r="F31" s="86" t="n"/>
+      <c r="F31" s="77" t="n"/>
       <c r="G31" s="77" t="n"/>
-      <c r="H31" s="86" t="n"/>
+      <c r="H31" s="77" t="n"/>
+      <c r="I31" s="78" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A7:I7"/>
+    <mergeCell ref="D27:I27"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D28:I28"/>
+    <mergeCell ref="D29:I29"/>
+    <mergeCell ref="D4:I4"/>
+    <mergeCell ref="D5:I5"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A31:I31"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="A24:I24"/>
+    <mergeCell ref="D25:I25"/>
+    <mergeCell ref="D26:I26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="47" min="1" max="1"/>
+    <col width="48" customWidth="1" style="47" min="2" max="2"/>
+    <col width="2" customWidth="1" style="47" min="3" max="3"/>
+    <col width="15" customWidth="1" style="47" min="4" max="4"/>
+    <col width="2" customWidth="1" style="47" min="5" max="5"/>
+    <col width="15" customWidth="1" style="47" min="6" max="6"/>
+    <col width="2" customWidth="1" style="47" min="7" max="7"/>
+    <col width="14" customWidth="1" style="47" min="8" max="8"/>
+    <col width="16" customWidth="1" style="47" min="9" max="9"/>
+    <col hidden="1" width="2" customWidth="1" style="47" min="10" max="10"/>
+    <col hidden="1" width="2" customWidth="1" style="47" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1" s="47">
+      <c r="A1" s="90" t="inlineStr">
+        <is>
+          <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — МОЙКА</t>
+        </is>
+      </c>
+      <c r="B1" s="75" t="n"/>
+      <c r="C1" s="75" t="n"/>
+      <c r="D1" s="75" t="n"/>
+      <c r="E1" s="75" t="n"/>
+      <c r="F1" s="75" t="n"/>
+      <c r="G1" s="75" t="n"/>
+      <c r="H1" s="75" t="n"/>
+      <c r="I1" s="75" t="n"/>
+    </row>
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
+        </is>
+      </c>
+      <c r="B2" s="76" t="n"/>
+      <c r="C2" s="76" t="n"/>
+      <c r="D2" s="76" t="n"/>
+      <c r="E2" s="76" t="n"/>
+      <c r="F2" s="76" t="n"/>
+      <c r="G2" s="76" t="n"/>
+      <c r="H2" s="76" t="n"/>
+      <c r="I2" s="76" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="47">
+      <c r="A3" s="64" t="n"/>
+      <c r="B3" s="65" t="inlineStr">
+        <is>
+          <t>АТЦ:</t>
+        </is>
+      </c>
+      <c r="C3" s="64" t="n"/>
+      <c r="D3" s="66" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="47">
+      <c r="A4" s="64" t="n"/>
+      <c r="B4" s="65" t="inlineStr">
+        <is>
+          <t>Неделя (авто):</t>
+        </is>
+      </c>
+      <c r="C4" s="64" t="n"/>
+      <c r="D4" s="66" t="n"/>
+      <c r="E4" s="77" t="n"/>
+      <c r="F4" s="77" t="n"/>
+      <c r="G4" s="77" t="n"/>
+      <c r="H4" s="77" t="n"/>
+      <c r="I4" s="78" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1" s="47">
+      <c r="A5" s="64" t="n"/>
+      <c r="B5" s="65" t="inlineStr">
+        <is>
+          <t>Руководитель (авто):</t>
+        </is>
+      </c>
+      <c r="C5" s="64" t="n"/>
+      <c r="D5" s="66" t="n"/>
+      <c r="E5" s="77" t="n"/>
+      <c r="F5" s="77" t="n"/>
+      <c r="G5" s="77" t="n"/>
+      <c r="H5" s="77" t="n"/>
+      <c r="I5" s="78" t="n"/>
+    </row>
+    <row r="6" ht="8" customHeight="1" s="47">
+      <c r="A6" s="55" t="n"/>
+      <c r="B6" s="55" t="n"/>
+      <c r="C6" s="55" t="n"/>
+      <c r="D6" s="55" t="n"/>
+      <c r="E6" s="55" t="n"/>
+      <c r="F6" s="55" t="n"/>
+      <c r="G6" s="55" t="n"/>
+      <c r="H6" s="55" t="n"/>
+      <c r="I6" s="55" t="n"/>
+    </row>
+    <row r="7" ht="33" customHeight="1" s="47">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1.  КЛЮЧЕВЫЕ ПОКАЗАТЕЛИ  [из 1С]</t>
+        </is>
+      </c>
+      <c r="B7" s="79" t="n"/>
+      <c r="C7" s="79" t="n"/>
+      <c r="D7" s="79" t="n"/>
+      <c r="E7" s="79" t="n"/>
+      <c r="F7" s="79" t="n"/>
+      <c r="G7" s="79" t="n"/>
+      <c r="H7" s="79" t="n"/>
+      <c r="I7" s="80" t="n"/>
+    </row>
+    <row r="8" ht="33" customHeight="1" s="47">
+      <c r="A8" s="68" t="n"/>
+      <c r="B8" s="68" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="C8" s="68" t="n"/>
+      <c r="D8" s="68" t="inlineStr">
+        <is>
+          <t>ПЛАН</t>
+        </is>
+      </c>
+      <c r="E8" s="68" t="n"/>
+      <c r="F8" s="68" t="inlineStr">
+        <is>
+          <t>ФАКТ (1С)</t>
+        </is>
+      </c>
+      <c r="G8" s="68" t="n"/>
+      <c r="H8" s="68" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I8" s="68" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="33" customHeight="1" s="47">
+      <c r="A9" s="69" t="n"/>
+      <c r="B9" s="69" t="inlineStr">
+        <is>
+          <t>Машин за неделю</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="n"/>
+      <c r="D9" s="81" t="n"/>
+      <c r="E9" s="70" t="n"/>
+      <c r="F9" s="81" t="n"/>
+      <c r="G9" s="70" t="n"/>
+      <c r="H9" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9&gt;0),F9/D9,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I9" s="70" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="33" customHeight="1" s="47">
+      <c r="A10" s="69" t="n"/>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>Выручка за неделю</t>
+        </is>
+      </c>
+      <c r="C10" s="70" t="n"/>
+      <c r="D10" s="81" t="n"/>
+      <c r="E10" s="70" t="n"/>
+      <c r="F10" s="81" t="n"/>
+      <c r="G10" s="70" t="n"/>
+      <c r="H10" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&gt;0),F10/D10,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I10" s="70" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="33" customHeight="1" s="47">
+      <c r="A11" s="69" t="n"/>
+      <c r="B11" s="69" t="inlineStr">
+        <is>
+          <t>Средний чек</t>
+        </is>
+      </c>
+      <c r="C11" s="70" t="n"/>
+      <c r="D11" s="81">
+        <f>IFERROR(D10/D9,"—")</f>
+        <v/>
+      </c>
+      <c r="E11" s="70" t="n"/>
+      <c r="F11" s="81">
+        <f>IFERROR(F10/F9,"—")</f>
+        <v/>
+      </c>
+      <c r="G11" s="70" t="n"/>
+      <c r="H11" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D11),ISNUMBER(F11),D11&gt;0),F11/D11,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I11" s="70" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="8" customHeight="1" s="47">
+      <c r="A12" s="55" t="n"/>
+      <c r="B12" s="55" t="n"/>
+      <c r="C12" s="55" t="n"/>
+      <c r="D12" s="83" t="n"/>
+      <c r="E12" s="55" t="n"/>
+      <c r="F12" s="83" t="n"/>
+      <c r="G12" s="55" t="n"/>
+      <c r="H12" s="83" t="n"/>
+      <c r="I12" s="55" t="n"/>
+    </row>
+    <row r="13" ht="33" customHeight="1" s="47">
+      <c r="A13" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2.  ДИНАМИКА ПО ДНЯМ  [из 1С]</t>
+        </is>
+      </c>
+      <c r="B13" s="79" t="n"/>
+      <c r="C13" s="79" t="n"/>
+      <c r="D13" s="79" t="n"/>
+      <c r="E13" s="79" t="n"/>
+      <c r="F13" s="79" t="n"/>
+      <c r="G13" s="79" t="n"/>
+      <c r="H13" s="79" t="n"/>
+      <c r="I13" s="80" t="n"/>
+    </row>
+    <row r="14" ht="33" customHeight="1" s="47">
+      <c r="A14" s="69" t="n"/>
+      <c r="B14" s="69" t="inlineStr">
+        <is>
+          <t>День</t>
+        </is>
+      </c>
+      <c r="C14" s="70" t="n"/>
+      <c r="D14" s="70" t="inlineStr">
+        <is>
+          <t>Машин</t>
+        </is>
+      </c>
+      <c r="E14" s="70" t="n"/>
+      <c r="F14" s="70" t="inlineStr">
+        <is>
+          <t>Выручка</t>
+        </is>
+      </c>
+      <c r="G14" s="70" t="n"/>
+      <c r="H14" s="70" t="inlineStr">
+        <is>
+          <t>Ср.чек</t>
+        </is>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>Операторов</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="33" customHeight="1" s="47">
+      <c r="A15" s="69" t="n"/>
+      <c r="B15" s="69" t="inlineStr">
+        <is>
+          <t>Пн</t>
+        </is>
+      </c>
+      <c r="C15" s="70" t="n"/>
+      <c r="D15" s="81" t="n"/>
+      <c r="E15" s="70" t="n"/>
+      <c r="F15" s="81" t="n"/>
+      <c r="G15" s="70" t="n"/>
+      <c r="H15" s="81">
+        <f>IFERROR(F15/D15,"—")</f>
+        <v/>
+      </c>
+      <c r="I15" s="70" t="n"/>
+    </row>
+    <row r="16" ht="33" customHeight="1" s="47">
+      <c r="A16" s="69" t="n"/>
+      <c r="B16" s="69" t="inlineStr">
+        <is>
+          <t>Вт</t>
+        </is>
+      </c>
+      <c r="C16" s="70" t="n"/>
+      <c r="D16" s="81" t="n"/>
+      <c r="E16" s="70" t="n"/>
+      <c r="F16" s="81" t="n"/>
+      <c r="G16" s="70" t="n"/>
+      <c r="H16" s="81">
+        <f>IFERROR(F16/D16,"—")</f>
+        <v/>
+      </c>
+      <c r="I16" s="70" t="n"/>
+    </row>
+    <row r="17" ht="33" customHeight="1" s="47">
+      <c r="A17" s="69" t="n"/>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>Ср</t>
+        </is>
+      </c>
+      <c r="C17" s="70" t="n"/>
+      <c r="D17" s="81" t="n"/>
+      <c r="E17" s="70" t="n"/>
+      <c r="F17" s="81" t="n"/>
+      <c r="G17" s="70" t="n"/>
+      <c r="H17" s="81">
+        <f>IFERROR(F17/D17,"—")</f>
+        <v/>
+      </c>
+      <c r="I17" s="70" t="n"/>
+    </row>
+    <row r="18" ht="33" customHeight="1" s="47">
+      <c r="A18" s="69" t="n"/>
+      <c r="B18" s="69" t="inlineStr">
+        <is>
+          <t>Чт</t>
+        </is>
+      </c>
+      <c r="C18" s="70" t="n"/>
+      <c r="D18" s="81" t="n"/>
+      <c r="E18" s="70" t="n"/>
+      <c r="F18" s="81" t="n"/>
+      <c r="G18" s="70" t="n"/>
+      <c r="H18" s="81">
+        <f>IFERROR(F18/D18,"—")</f>
+        <v/>
+      </c>
+      <c r="I18" s="70" t="n"/>
+    </row>
+    <row r="19" ht="33" customHeight="1" s="47">
+      <c r="A19" s="69" t="n"/>
+      <c r="B19" s="69" t="inlineStr">
+        <is>
+          <t>Пт</t>
+        </is>
+      </c>
+      <c r="C19" s="70" t="n"/>
+      <c r="D19" s="81" t="n"/>
+      <c r="E19" s="70" t="n"/>
+      <c r="F19" s="81" t="n"/>
+      <c r="G19" s="70" t="n"/>
+      <c r="H19" s="81">
+        <f>IFERROR(F19/D19,"—")</f>
+        <v/>
+      </c>
+      <c r="I19" s="70" t="n"/>
+    </row>
+    <row r="20" ht="33" customHeight="1" s="47">
+      <c r="A20" s="69" t="n"/>
+      <c r="B20" s="69" t="inlineStr">
+        <is>
+          <t>Сб</t>
+        </is>
+      </c>
+      <c r="C20" s="70" t="n"/>
+      <c r="D20" s="81" t="n"/>
+      <c r="E20" s="70" t="n"/>
+      <c r="F20" s="81" t="n"/>
+      <c r="G20" s="70" t="n"/>
+      <c r="H20" s="81">
+        <f>IFERROR(F20/D20,"—")</f>
+        <v/>
+      </c>
+      <c r="I20" s="70" t="n"/>
+    </row>
+    <row r="21" ht="33" customHeight="1" s="47">
+      <c r="A21" s="69" t="n"/>
+      <c r="B21" s="69" t="inlineStr">
+        <is>
+          <t>Вс</t>
+        </is>
+      </c>
+      <c r="C21" s="70" t="n"/>
+      <c r="D21" s="81" t="n"/>
+      <c r="E21" s="70" t="n"/>
+      <c r="F21" s="81" t="n"/>
+      <c r="G21" s="70" t="n"/>
+      <c r="H21" s="81">
+        <f>IFERROR(F21/D21,"—")</f>
+        <v/>
+      </c>
+      <c r="I21" s="70" t="n"/>
+    </row>
+    <row r="22" ht="33" customHeight="1" s="47">
+      <c r="A22" s="69" t="n"/>
+      <c r="B22" s="69" t="inlineStr">
+        <is>
+          <t>ИТОГО</t>
+        </is>
+      </c>
+      <c r="C22" s="70" t="n"/>
+      <c r="D22" s="81">
+        <f>SUM(D15:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="70" t="n"/>
+      <c r="F22" s="81">
+        <f>SUM(F15:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="70" t="n"/>
+      <c r="H22" s="81">
+        <f>IFERROR(F22/D22,"—")</f>
+        <v/>
+      </c>
+      <c r="I22" s="70" t="n"/>
+    </row>
+    <row r="23" ht="8" customHeight="1" s="47">
+      <c r="A23" s="55" t="n"/>
+      <c r="B23" s="55" t="n"/>
+      <c r="C23" s="55" t="n"/>
+      <c r="D23" s="83" t="n"/>
+      <c r="E23" s="55" t="n"/>
+      <c r="F23" s="83" t="n"/>
+      <c r="G23" s="55" t="n"/>
+      <c r="H23" s="83" t="n"/>
+      <c r="I23" s="55" t="n"/>
+    </row>
+    <row r="24" ht="33" customHeight="1" s="47">
+      <c r="A24" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3.  КОММЕНТАРИЙ РУКОВОДИТЕЛЯ  [вручную]</t>
+        </is>
+      </c>
+      <c r="B24" s="79" t="n"/>
+      <c r="C24" s="79" t="n"/>
+      <c r="D24" s="79" t="n"/>
+      <c r="E24" s="79" t="n"/>
+      <c r="F24" s="79" t="n"/>
+      <c r="G24" s="79" t="n"/>
+      <c r="H24" s="79" t="n"/>
+      <c r="I24" s="80" t="n"/>
+    </row>
+    <row r="25" ht="33" customHeight="1" s="47">
+      <c r="A25" s="69" t="n"/>
+      <c r="B25" s="69" t="inlineStr">
+        <is>
+          <t>Вопрос</t>
+        </is>
+      </c>
+      <c r="C25" s="70" t="n"/>
+      <c r="D25" s="70" t="inlineStr">
+        <is>
+          <t>Ответ / комментарий</t>
+        </is>
+      </c>
+      <c r="E25" s="77" t="n"/>
+      <c r="F25" s="77" t="n"/>
+      <c r="G25" s="77" t="n"/>
+      <c r="H25" s="77" t="n"/>
+      <c r="I25" s="78" t="n"/>
+    </row>
+    <row r="26" ht="33" customHeight="1" s="47">
+      <c r="A26" s="69" t="n"/>
+      <c r="B26" s="69" t="inlineStr">
+        <is>
+          <t>Что повлияло на трафик за неделю?</t>
+        </is>
+      </c>
+      <c r="C26" s="70" t="n"/>
+      <c r="D26" s="70" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E26" s="77" t="n"/>
+      <c r="F26" s="77" t="n"/>
+      <c r="G26" s="77" t="n"/>
+      <c r="H26" s="77" t="n"/>
+      <c r="I26" s="78" t="n"/>
+    </row>
+    <row r="27" ht="33" customHeight="1" s="47">
+      <c r="A27" s="69" t="n"/>
+      <c r="B27" s="69" t="inlineStr">
+        <is>
+          <t>Проблемы с оборудованием/химией</t>
+        </is>
+      </c>
+      <c r="C27" s="70" t="n"/>
+      <c r="D27" s="70" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E27" s="77" t="n"/>
+      <c r="F27" s="77" t="n"/>
+      <c r="G27" s="77" t="n"/>
+      <c r="H27" s="77" t="n"/>
+      <c r="I27" s="78" t="n"/>
+    </row>
+    <row r="28" ht="33" customHeight="1" s="47">
+      <c r="A28" s="69" t="n"/>
+      <c r="B28" s="69" t="inlineStr">
+        <is>
+          <t>Задачи на следующую неделю</t>
+        </is>
+      </c>
+      <c r="C28" s="70" t="n"/>
+      <c r="D28" s="70" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E28" s="77" t="n"/>
+      <c r="F28" s="77" t="n"/>
+      <c r="G28" s="77" t="n"/>
+      <c r="H28" s="77" t="n"/>
+      <c r="I28" s="78" t="n"/>
+    </row>
+    <row r="29" ht="33" customHeight="1" s="47">
+      <c r="A29" s="69" t="n"/>
+      <c r="B29" s="69" t="inlineStr">
+        <is>
+          <t>Что требует решения ГД?</t>
+        </is>
+      </c>
+      <c r="C29" s="70" t="n"/>
+      <c r="D29" s="70" t="inlineStr">
+        <is>
+          <t>введите комментарий...</t>
+        </is>
+      </c>
+      <c r="E29" s="77" t="n"/>
+      <c r="F29" s="77" t="n"/>
+      <c r="G29" s="77" t="n"/>
+      <c r="H29" s="77" t="n"/>
+      <c r="I29" s="78" t="n"/>
+    </row>
+    <row r="30" ht="8" customHeight="1" s="47">
+      <c r="A30" s="55" t="n"/>
+      <c r="B30" s="55" t="n"/>
+      <c r="C30" s="55" t="n"/>
+      <c r="D30" s="83" t="n"/>
+      <c r="E30" s="55" t="n"/>
+      <c r="F30" s="83" t="n"/>
+      <c r="G30" s="55" t="n"/>
+      <c r="H30" s="83" t="n"/>
+      <c r="I30" s="55" t="n"/>
+    </row>
+    <row r="31" ht="33" customHeight="1" s="47">
+      <c r="A31" s="69" t="inlineStr">
+        <is>
+          <t>🤖 Данные 1С — авто | 🖊 Комментарии — руководитель до 11:00 пн | Битрикс24</t>
+        </is>
+      </c>
+      <c r="B31" s="77" t="n"/>
+      <c r="C31" s="77" t="n"/>
+      <c r="D31" s="77" t="n"/>
+      <c r="E31" s="77" t="n"/>
+      <c r="F31" s="77" t="n"/>
+      <c r="G31" s="77" t="n"/>
+      <c r="H31" s="77" t="n"/>
       <c r="I31" s="78" t="n"/>
     </row>
   </sheetData>
@@ -2901,6 +2894,553 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="47" min="1" max="1"/>
+    <col width="48" customWidth="1" style="47" min="2" max="2"/>
+    <col width="2" customWidth="1" style="47" min="3" max="3"/>
+    <col width="15" customWidth="1" style="47" min="4" max="4"/>
+    <col width="2" customWidth="1" style="47" min="5" max="5"/>
+    <col width="15" customWidth="1" style="47" min="6" max="6"/>
+    <col width="2" customWidth="1" style="47" min="7" max="7"/>
+    <col width="14" customWidth="1" style="47" min="8" max="8"/>
+    <col width="16" customWidth="1" style="47" min="9" max="9"/>
+    <col hidden="1" width="2" customWidth="1" style="47" min="10" max="10"/>
+    <col hidden="1" width="2" customWidth="1" style="47" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1" s="47">
+      <c r="A1" s="90" t="inlineStr">
+        <is>
+          <t>ЕЖЕДНЕВНЫЙ ОТЧЁТ — АРСЕНАЛ  |  Данные из 1С</t>
+        </is>
+      </c>
+      <c r="B1" s="75" t="n"/>
+      <c r="C1" s="75" t="n"/>
+      <c r="D1" s="75" t="n"/>
+      <c r="E1" s="75" t="n"/>
+      <c r="F1" s="75" t="n"/>
+      <c r="G1" s="75" t="n"/>
+      <c r="H1" s="75" t="n"/>
+      <c r="I1" s="75" t="n"/>
+    </row>
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
+        </is>
+      </c>
+      <c r="B2" s="76" t="n"/>
+      <c r="C2" s="76" t="n"/>
+      <c r="D2" s="76" t="n"/>
+      <c r="E2" s="76" t="n"/>
+      <c r="F2" s="76" t="n"/>
+      <c r="G2" s="76" t="n"/>
+      <c r="H2" s="76" t="n"/>
+      <c r="I2" s="76" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1" s="47">
+      <c r="A3" s="64" t="n"/>
+      <c r="B3" s="65" t="inlineStr">
+        <is>
+          <t>АТЦ:</t>
+        </is>
+      </c>
+      <c r="C3" s="64" t="n"/>
+      <c r="D3" s="66" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1" s="47">
+      <c r="A4" s="64" t="n"/>
+      <c r="B4" s="65" t="inlineStr">
+        <is>
+          <t>Дата (авто):</t>
+        </is>
+      </c>
+      <c r="C4" s="64" t="n"/>
+      <c r="D4" s="66" t="n"/>
+      <c r="E4" s="77" t="n"/>
+      <c r="F4" s="77" t="n"/>
+      <c r="G4" s="77" t="n"/>
+      <c r="H4" s="77" t="n"/>
+      <c r="I4" s="78" t="n"/>
+    </row>
+    <row r="5" ht="26" customHeight="1" s="47">
+      <c r="A5" s="64" t="n"/>
+      <c r="B5" s="65" t="n"/>
+      <c r="C5" s="64" t="n"/>
+      <c r="D5" s="66" t="n"/>
+      <c r="E5" s="66" t="n"/>
+      <c r="F5" s="66" t="n"/>
+      <c r="G5" s="66" t="n"/>
+      <c r="H5" s="66" t="n"/>
+      <c r="I5" s="66" t="n"/>
+    </row>
+    <row r="6" ht="33" customHeight="1" s="47">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ВЫРАБОТКА</t>
+        </is>
+      </c>
+      <c r="B6" s="79" t="n"/>
+      <c r="C6" s="79" t="n"/>
+      <c r="D6" s="79" t="n"/>
+      <c r="E6" s="79" t="n"/>
+      <c r="F6" s="79" t="n"/>
+      <c r="G6" s="79" t="n"/>
+      <c r="H6" s="79" t="n"/>
+      <c r="I6" s="80" t="n"/>
+    </row>
+    <row r="7" ht="33" customHeight="1" s="47">
+      <c r="A7" s="68" t="n"/>
+      <c r="B7" s="68" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="C7" s="68" t="n"/>
+      <c r="D7" s="68" t="inlineStr">
+        <is>
+          <t>ПЛАН</t>
+        </is>
+      </c>
+      <c r="E7" s="68" t="n"/>
+      <c r="F7" s="68" t="inlineStr">
+        <is>
+          <t>ФАКТ (1С)</t>
+        </is>
+      </c>
+      <c r="G7" s="68" t="n"/>
+      <c r="H7" s="68" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I7" s="68" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="33" customHeight="1" s="47">
+      <c r="A8" s="69" t="n"/>
+      <c r="B8" s="69" t="inlineStr">
+        <is>
+          <t>Нормочасы за день — общая выработка</t>
+        </is>
+      </c>
+      <c r="C8" s="70" t="n"/>
+      <c r="D8" s="81" t="n"/>
+      <c r="E8" s="70" t="n"/>
+      <c r="F8" s="81" t="n"/>
+      <c r="G8" s="70" t="n"/>
+      <c r="H8" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D8),ISNUMBER(F8),D8&gt;0),F8/D8,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I8" s="70" t="inlineStr">
+        <is>
+          <t>нч</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="33" customHeight="1" s="47">
+      <c r="A9" s="69" t="n"/>
+      <c r="B9" s="69" t="inlineStr">
+        <is>
+          <t>Выработка на 1 мастера (нч/чел.)</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="n"/>
+      <c r="D9" s="81" t="n"/>
+      <c r="E9" s="70" t="n"/>
+      <c r="F9" s="81" t="n"/>
+      <c r="G9" s="70" t="n"/>
+      <c r="H9" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9&gt;0),F9/D9,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I9" s="70" t="inlineStr">
+        <is>
+          <t>нч/чел</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="33" customHeight="1" s="47">
+      <c r="A10" s="69" t="n"/>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>Закрыто ЗН за день</t>
+        </is>
+      </c>
+      <c r="C10" s="70" t="n"/>
+      <c r="D10" s="81" t="n"/>
+      <c r="E10" s="70" t="n"/>
+      <c r="F10" s="81" t="n"/>
+      <c r="G10" s="70" t="n"/>
+      <c r="H10" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&gt;0),F10/D10,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I10" s="70" t="inlineStr">
+        <is>
+          <t>шт.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="8" customHeight="1" s="47">
+      <c r="A11" s="55" t="n"/>
+      <c r="B11" s="55" t="n"/>
+      <c r="C11" s="55" t="n"/>
+      <c r="D11" s="83" t="n"/>
+      <c r="E11" s="55" t="n"/>
+      <c r="F11" s="83" t="n"/>
+      <c r="G11" s="55" t="n"/>
+      <c r="H11" s="83" t="n"/>
+      <c r="I11" s="55" t="n"/>
+    </row>
+    <row r="12" ht="33" customHeight="1" s="47">
+      <c r="A12" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ФИНАНСЫ</t>
+        </is>
+      </c>
+      <c r="B12" s="79" t="n"/>
+      <c r="C12" s="79" t="n"/>
+      <c r="D12" s="79" t="n"/>
+      <c r="E12" s="79" t="n"/>
+      <c r="F12" s="79" t="n"/>
+      <c r="G12" s="79" t="n"/>
+      <c r="H12" s="79" t="n"/>
+      <c r="I12" s="80" t="n"/>
+    </row>
+    <row r="13" ht="33" customHeight="1" s="47">
+      <c r="A13" s="68" t="n"/>
+      <c r="B13" s="68" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="C13" s="68" t="n"/>
+      <c r="D13" s="68" t="inlineStr">
+        <is>
+          <t>ПЛАН</t>
+        </is>
+      </c>
+      <c r="E13" s="68" t="n"/>
+      <c r="F13" s="68" t="inlineStr">
+        <is>
+          <t>ФАКТ (1С)</t>
+        </is>
+      </c>
+      <c r="G13" s="68" t="n"/>
+      <c r="H13" s="68" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="I13" s="68" t="inlineStr">
+        <is>
+          <t>Ед.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="33" customHeight="1" s="47">
+      <c r="A14" s="69" t="n"/>
+      <c r="B14" s="69" t="inlineStr">
+        <is>
+          <t>Выручка за день</t>
+        </is>
+      </c>
+      <c r="C14" s="70" t="n"/>
+      <c r="D14" s="81" t="n"/>
+      <c r="E14" s="70" t="n"/>
+      <c r="F14" s="81" t="n"/>
+      <c r="G14" s="70" t="n"/>
+      <c r="H14" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D14),ISNUMBER(F14),D14&gt;0),F14/D14,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I14" s="70" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="33" customHeight="1" s="47">
+      <c r="A15" s="69" t="n"/>
+      <c r="B15" s="69" t="inlineStr">
+        <is>
+          <t>Себестоимость ЗЧ</t>
+        </is>
+      </c>
+      <c r="C15" s="70" t="n"/>
+      <c r="D15" s="81" t="n"/>
+      <c r="E15" s="70" t="n"/>
+      <c r="F15" s="81" t="n"/>
+      <c r="G15" s="70" t="n"/>
+      <c r="H15" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D15),ISNUMBER(F15),D15&gt;0),F15/D15,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I15" s="70" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="33" customHeight="1" s="47">
+      <c r="A16" s="69" t="n"/>
+      <c r="B16" s="69" t="inlineStr">
+        <is>
+          <t>Маржа (Выручка − Себест. ЗЧ)</t>
+        </is>
+      </c>
+      <c r="C16" s="70" t="n"/>
+      <c r="D16" s="81">
+        <f>IFERROR(D14-D15,"—")</f>
+        <v/>
+      </c>
+      <c r="E16" s="70" t="n"/>
+      <c r="F16" s="81">
+        <f>IFERROR(F14-F15,"—")</f>
+        <v/>
+      </c>
+      <c r="G16" s="70" t="n"/>
+      <c r="H16" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D16),ISNUMBER(F16),D16&gt;0),F16/D16,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I16" s="70" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="33" customHeight="1" s="47">
+      <c r="A17" s="69" t="n"/>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>Маржинальность</t>
+        </is>
+      </c>
+      <c r="C17" s="70" t="n"/>
+      <c r="D17" s="82">
+        <f>IFERROR(D16/D14,"—")</f>
+        <v/>
+      </c>
+      <c r="E17" s="70" t="n"/>
+      <c r="F17" s="82">
+        <f>IFERROR(F16/F14,"—")</f>
+        <v/>
+      </c>
+      <c r="G17" s="70" t="n"/>
+      <c r="H17" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D17),ISNUMBER(F17),D17&gt;0),F17/D17,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I17" s="70" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="33" customHeight="1" s="47">
+      <c r="A18" s="69" t="n"/>
+      <c r="B18" s="69" t="inlineStr">
+        <is>
+          <t>Средний чек (руб./ЗН)</t>
+        </is>
+      </c>
+      <c r="C18" s="70" t="n"/>
+      <c r="D18" s="81">
+        <f>IFERROR(D14/D10,"—")</f>
+        <v/>
+      </c>
+      <c r="E18" s="70" t="n"/>
+      <c r="F18" s="81">
+        <f>IFERROR(F14/F10,"—")</f>
+        <v/>
+      </c>
+      <c r="G18" s="70" t="n"/>
+      <c r="H18" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D18),ISNUMBER(F18),D18&gt;0),F18/D18,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I18" s="70" t="inlineStr">
+        <is>
+          <t>руб.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="33" customHeight="1" s="47">
+      <c r="A19" s="69" t="n"/>
+      <c r="B19" s="69" t="inlineStr">
+        <is>
+          <t>Наценка на ЗЧ</t>
+        </is>
+      </c>
+      <c r="C19" s="70" t="n"/>
+      <c r="D19" s="82" t="n"/>
+      <c r="E19" s="70" t="n"/>
+      <c r="F19" s="82" t="n"/>
+      <c r="G19" s="70" t="n"/>
+      <c r="H19" s="82">
+        <f>IFERROR(IF(AND(ISNUMBER(D19),ISNUMBER(F19),D19&gt;0),F19/D19,"—"),"—")</f>
+        <v/>
+      </c>
+      <c r="I19" s="70" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="8" customHeight="1" s="47">
+      <c r="A20" s="55" t="n"/>
+      <c r="B20" s="55" t="n"/>
+      <c r="C20" s="55" t="n"/>
+      <c r="D20" s="83" t="n"/>
+      <c r="E20" s="55" t="n"/>
+      <c r="F20" s="83" t="n"/>
+      <c r="G20" s="55" t="n"/>
+      <c r="H20" s="83" t="n"/>
+      <c r="I20" s="55" t="n"/>
+    </row>
+    <row r="21" ht="33" customHeight="1" s="47">
+      <c r="A21" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  СНАБЖЕНИЕ (из 1С)</t>
+        </is>
+      </c>
+      <c r="B21" s="79" t="n"/>
+      <c r="C21" s="79" t="n"/>
+      <c r="D21" s="79" t="n"/>
+      <c r="E21" s="79" t="n"/>
+      <c r="F21" s="79" t="n"/>
+      <c r="G21" s="79" t="n"/>
+      <c r="H21" s="79" t="n"/>
+      <c r="I21" s="80" t="n"/>
+    </row>
+    <row r="22" ht="33" customHeight="1" s="47">
+      <c r="A22" s="68" t="n"/>
+      <c r="B22" s="68" t="inlineStr">
+        <is>
+          <t>Показатель</t>
+        </is>
+      </c>
+      <c r="C22" s="68" t="n"/>
+      <c r="D22" s="68" t="inlineStr">
+        <is>
+          <t>Значение (1С)</t>
+        </is>
+      </c>
+      <c r="E22" s="77" t="n"/>
+      <c r="F22" s="78" t="n"/>
+      <c r="G22" s="68" t="n"/>
+      <c r="H22" s="68" t="inlineStr">
+        <is>
+          <t>Норма</t>
+        </is>
+      </c>
+      <c r="I22" s="78" t="n"/>
+    </row>
+    <row r="23" ht="33" customHeight="1" s="47">
+      <c r="A23" s="69" t="n"/>
+      <c r="B23" s="69" t="inlineStr">
+        <is>
+          <t>Незакрытые ЗН старше 1 дня (шт.)</t>
+        </is>
+      </c>
+      <c r="C23" s="70" t="n"/>
+      <c r="D23" s="81" t="n"/>
+      <c r="E23" s="77" t="n"/>
+      <c r="F23" s="78" t="n"/>
+      <c r="G23" s="70" t="n"/>
+      <c r="H23" s="70" t="inlineStr">
+        <is>
+          <t>Цель: 0</t>
+        </is>
+      </c>
+      <c r="I23" s="78" t="n"/>
+    </row>
+    <row r="24" ht="33" customHeight="1" s="47">
+      <c r="A24" s="69" t="n"/>
+      <c r="B24" s="69" t="inlineStr">
+        <is>
+          <t>ЗН без движения &gt; 2 дней (шт.)</t>
+        </is>
+      </c>
+      <c r="C24" s="70" t="n"/>
+      <c r="D24" s="81" t="n"/>
+      <c r="E24" s="77" t="n"/>
+      <c r="F24" s="78" t="n"/>
+      <c r="G24" s="70" t="n"/>
+      <c r="H24" s="70" t="inlineStr">
+        <is>
+          <t>Цель: 0</t>
+        </is>
+      </c>
+      <c r="I24" s="78" t="n"/>
+    </row>
+    <row r="25" ht="8" customHeight="1" s="47">
+      <c r="A25" s="55" t="n"/>
+      <c r="B25" s="55" t="n"/>
+      <c r="C25" s="55" t="n"/>
+      <c r="D25" s="83" t="n"/>
+      <c r="E25" s="55" t="n"/>
+      <c r="F25" s="83" t="n"/>
+      <c r="G25" s="55" t="n"/>
+      <c r="H25" s="83" t="n"/>
+      <c r="I25" s="55" t="n"/>
+    </row>
+    <row r="26" ht="33" customHeight="1" s="47">
+      <c r="A26" s="69" t="inlineStr">
+        <is>
+          <t>🤖 Генерируется автоматически в 11:00 | Данные: 1С Альфа-Авто | Отправка: Битрикс24</t>
+        </is>
+      </c>
+      <c r="B26" s="77" t="n"/>
+      <c r="C26" s="77" t="n"/>
+      <c r="D26" s="77" t="n"/>
+      <c r="E26" s="77" t="n"/>
+      <c r="F26" s="77" t="n"/>
+      <c r="G26" s="77" t="n"/>
+      <c r="H26" s="77" t="n"/>
+      <c r="I26" s="78" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D4:I4"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="D22:F22"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="A6:I6"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A21:I21"/>
+    <mergeCell ref="D24:F24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
@@ -2918,7 +3458,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — АРСЕНАЛ</t>
         </is>
@@ -2932,8 +3472,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -3134,11 +3674,11 @@
       </c>
       <c r="B13" s="79" t="n"/>
       <c r="C13" s="79" t="n"/>
-      <c r="D13" s="84" t="n"/>
+      <c r="D13" s="79" t="n"/>
       <c r="E13" s="79" t="n"/>
-      <c r="F13" s="84" t="n"/>
+      <c r="F13" s="79" t="n"/>
       <c r="G13" s="79" t="n"/>
-      <c r="H13" s="84" t="n"/>
+      <c r="H13" s="79" t="n"/>
       <c r="I13" s="80" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
@@ -3341,11 +3881,11 @@
       </c>
       <c r="B22" s="79" t="n"/>
       <c r="C22" s="79" t="n"/>
-      <c r="D22" s="84" t="n"/>
+      <c r="D22" s="79" t="n"/>
       <c r="E22" s="79" t="n"/>
-      <c r="F22" s="84" t="n"/>
+      <c r="F22" s="79" t="n"/>
       <c r="G22" s="79" t="n"/>
-      <c r="H22" s="84" t="n"/>
+      <c r="H22" s="79" t="n"/>
       <c r="I22" s="80" t="n"/>
     </row>
     <row r="23" ht="33" customHeight="1" s="47">
@@ -3551,11 +4091,11 @@
       </c>
       <c r="B33" s="79" t="n"/>
       <c r="C33" s="79" t="n"/>
-      <c r="D33" s="84" t="n"/>
+      <c r="D33" s="79" t="n"/>
       <c r="E33" s="79" t="n"/>
-      <c r="F33" s="84" t="n"/>
+      <c r="F33" s="79" t="n"/>
       <c r="G33" s="79" t="n"/>
-      <c r="H33" s="84" t="n"/>
+      <c r="H33" s="79" t="n"/>
       <c r="I33" s="80" t="n"/>
     </row>
     <row r="34" ht="33" customHeight="1" s="47">
@@ -3572,9 +4112,9 @@
         </is>
       </c>
       <c r="E34" s="77" t="n"/>
-      <c r="F34" s="86" t="n"/>
+      <c r="F34" s="77" t="n"/>
       <c r="G34" s="77" t="n"/>
-      <c r="H34" s="86" t="n"/>
+      <c r="H34" s="77" t="n"/>
       <c r="I34" s="78" t="n"/>
     </row>
     <row r="35" ht="33" customHeight="1" s="47">
@@ -3591,9 +4131,9 @@
         </is>
       </c>
       <c r="E35" s="77" t="n"/>
-      <c r="F35" s="86" t="n"/>
+      <c r="F35" s="77" t="n"/>
       <c r="G35" s="77" t="n"/>
-      <c r="H35" s="86" t="n"/>
+      <c r="H35" s="77" t="n"/>
       <c r="I35" s="78" t="n"/>
     </row>
     <row r="36" ht="33" customHeight="1" s="47">
@@ -3610,9 +4150,9 @@
         </is>
       </c>
       <c r="E36" s="77" t="n"/>
-      <c r="F36" s="86" t="n"/>
+      <c r="F36" s="77" t="n"/>
       <c r="G36" s="77" t="n"/>
-      <c r="H36" s="86" t="n"/>
+      <c r="H36" s="77" t="n"/>
       <c r="I36" s="78" t="n"/>
     </row>
     <row r="37" ht="33" customHeight="1" s="47">
@@ -3629,9 +4169,9 @@
         </is>
       </c>
       <c r="E37" s="77" t="n"/>
-      <c r="F37" s="86" t="n"/>
+      <c r="F37" s="77" t="n"/>
       <c r="G37" s="77" t="n"/>
-      <c r="H37" s="86" t="n"/>
+      <c r="H37" s="77" t="n"/>
       <c r="I37" s="78" t="n"/>
     </row>
     <row r="38" ht="33" customHeight="1" s="47">
@@ -3648,9 +4188,9 @@
         </is>
       </c>
       <c r="E38" s="77" t="n"/>
-      <c r="F38" s="86" t="n"/>
+      <c r="F38" s="77" t="n"/>
       <c r="G38" s="77" t="n"/>
-      <c r="H38" s="86" t="n"/>
+      <c r="H38" s="77" t="n"/>
       <c r="I38" s="78" t="n"/>
     </row>
     <row r="39" ht="33" customHeight="1" s="47">
@@ -3667,9 +4207,9 @@
         </is>
       </c>
       <c r="E39" s="77" t="n"/>
-      <c r="F39" s="86" t="n"/>
+      <c r="F39" s="77" t="n"/>
       <c r="G39" s="77" t="n"/>
-      <c r="H39" s="86" t="n"/>
+      <c r="H39" s="77" t="n"/>
       <c r="I39" s="78" t="n"/>
     </row>
     <row r="40" ht="33" customHeight="1" s="47">
@@ -3686,9 +4226,9 @@
         </is>
       </c>
       <c r="E40" s="77" t="n"/>
-      <c r="F40" s="86" t="n"/>
+      <c r="F40" s="77" t="n"/>
       <c r="G40" s="77" t="n"/>
-      <c r="H40" s="86" t="n"/>
+      <c r="H40" s="77" t="n"/>
       <c r="I40" s="78" t="n"/>
     </row>
     <row r="41" ht="8" customHeight="1" s="47">
@@ -3710,11 +4250,11 @@
       </c>
       <c r="B42" s="77" t="n"/>
       <c r="C42" s="77" t="n"/>
-      <c r="D42" s="86" t="n"/>
+      <c r="D42" s="77" t="n"/>
       <c r="E42" s="77" t="n"/>
-      <c r="F42" s="86" t="n"/>
+      <c r="F42" s="77" t="n"/>
       <c r="G42" s="77" t="n"/>
-      <c r="H42" s="86" t="n"/>
+      <c r="H42" s="77" t="n"/>
       <c r="I42" s="78" t="n"/>
     </row>
   </sheetData>
@@ -3742,7 +4282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3765,7 +4305,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕДНЕВНЫЙ ОТЧЁТ — РЕФ.СЕРВИС  |  Данные из 1С</t>
         </is>
@@ -3779,8 +4319,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -3966,11 +4506,11 @@
       </c>
       <c r="B12" s="79" t="n"/>
       <c r="C12" s="79" t="n"/>
-      <c r="D12" s="84" t="n"/>
+      <c r="D12" s="79" t="n"/>
       <c r="E12" s="79" t="n"/>
-      <c r="F12" s="84" t="n"/>
+      <c r="F12" s="79" t="n"/>
       <c r="G12" s="79" t="n"/>
-      <c r="H12" s="84" t="n"/>
+      <c r="H12" s="79" t="n"/>
       <c r="I12" s="80" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1" s="47">
@@ -4173,11 +4713,11 @@
       </c>
       <c r="B21" s="79" t="n"/>
       <c r="C21" s="79" t="n"/>
-      <c r="D21" s="84" t="n"/>
+      <c r="D21" s="79" t="n"/>
       <c r="E21" s="79" t="n"/>
-      <c r="F21" s="84" t="n"/>
+      <c r="F21" s="79" t="n"/>
       <c r="G21" s="79" t="n"/>
-      <c r="H21" s="84" t="n"/>
+      <c r="H21" s="79" t="n"/>
       <c r="I21" s="80" t="n"/>
     </row>
     <row r="22" ht="33" customHeight="1" s="47">
@@ -4194,7 +4734,7 @@
         </is>
       </c>
       <c r="E22" s="77" t="n"/>
-      <c r="F22" s="85" t="n"/>
+      <c r="F22" s="78" t="n"/>
       <c r="G22" s="68" t="n"/>
       <c r="H22" s="68" t="inlineStr">
         <is>
@@ -4213,7 +4753,7 @@
       <c r="C23" s="70" t="n"/>
       <c r="D23" s="81" t="n"/>
       <c r="E23" s="77" t="n"/>
-      <c r="F23" s="85" t="n"/>
+      <c r="F23" s="78" t="n"/>
       <c r="G23" s="70" t="n"/>
       <c r="H23" s="70" t="inlineStr">
         <is>
@@ -4232,7 +4772,7 @@
       <c r="C24" s="70" t="n"/>
       <c r="D24" s="81" t="n"/>
       <c r="E24" s="77" t="n"/>
-      <c r="F24" s="85" t="n"/>
+      <c r="F24" s="78" t="n"/>
       <c r="G24" s="70" t="n"/>
       <c r="H24" s="70" t="inlineStr">
         <is>
@@ -4260,11 +4800,11 @@
       </c>
       <c r="B26" s="77" t="n"/>
       <c r="C26" s="77" t="n"/>
-      <c r="D26" s="86" t="n"/>
+      <c r="D26" s="77" t="n"/>
       <c r="E26" s="77" t="n"/>
-      <c r="F26" s="86" t="n"/>
+      <c r="F26" s="77" t="n"/>
       <c r="G26" s="77" t="n"/>
-      <c r="H26" s="86" t="n"/>
+      <c r="H26" s="77" t="n"/>
       <c r="I26" s="78" t="n"/>
     </row>
   </sheetData>
@@ -4289,7 +4829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4312,7 +4852,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — РЕФ.СЕРВИС</t>
         </is>
@@ -4326,8 +4866,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -4528,11 +5068,11 @@
       </c>
       <c r="B13" s="79" t="n"/>
       <c r="C13" s="79" t="n"/>
-      <c r="D13" s="84" t="n"/>
+      <c r="D13" s="79" t="n"/>
       <c r="E13" s="79" t="n"/>
-      <c r="F13" s="84" t="n"/>
+      <c r="F13" s="79" t="n"/>
       <c r="G13" s="79" t="n"/>
-      <c r="H13" s="84" t="n"/>
+      <c r="H13" s="79" t="n"/>
       <c r="I13" s="80" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
@@ -4735,11 +5275,11 @@
       </c>
       <c r="B22" s="79" t="n"/>
       <c r="C22" s="79" t="n"/>
-      <c r="D22" s="84" t="n"/>
+      <c r="D22" s="79" t="n"/>
       <c r="E22" s="79" t="n"/>
-      <c r="F22" s="84" t="n"/>
+      <c r="F22" s="79" t="n"/>
       <c r="G22" s="79" t="n"/>
-      <c r="H22" s="84" t="n"/>
+      <c r="H22" s="79" t="n"/>
       <c r="I22" s="80" t="n"/>
     </row>
     <row r="23" ht="33" customHeight="1" s="47">
@@ -4945,11 +5485,11 @@
       </c>
       <c r="B33" s="79" t="n"/>
       <c r="C33" s="79" t="n"/>
-      <c r="D33" s="84" t="n"/>
+      <c r="D33" s="79" t="n"/>
       <c r="E33" s="79" t="n"/>
-      <c r="F33" s="84" t="n"/>
+      <c r="F33" s="79" t="n"/>
       <c r="G33" s="79" t="n"/>
-      <c r="H33" s="84" t="n"/>
+      <c r="H33" s="79" t="n"/>
       <c r="I33" s="80" t="n"/>
     </row>
     <row r="34" ht="33" customHeight="1" s="47">
@@ -4966,9 +5506,9 @@
         </is>
       </c>
       <c r="E34" s="77" t="n"/>
-      <c r="F34" s="86" t="n"/>
+      <c r="F34" s="77" t="n"/>
       <c r="G34" s="77" t="n"/>
-      <c r="H34" s="86" t="n"/>
+      <c r="H34" s="77" t="n"/>
       <c r="I34" s="78" t="n"/>
     </row>
     <row r="35" ht="33" customHeight="1" s="47">
@@ -4985,9 +5525,9 @@
         </is>
       </c>
       <c r="E35" s="77" t="n"/>
-      <c r="F35" s="86" t="n"/>
+      <c r="F35" s="77" t="n"/>
       <c r="G35" s="77" t="n"/>
-      <c r="H35" s="86" t="n"/>
+      <c r="H35" s="77" t="n"/>
       <c r="I35" s="78" t="n"/>
     </row>
     <row r="36" ht="33" customHeight="1" s="47">
@@ -5004,9 +5544,9 @@
         </is>
       </c>
       <c r="E36" s="77" t="n"/>
-      <c r="F36" s="86" t="n"/>
+      <c r="F36" s="77" t="n"/>
       <c r="G36" s="77" t="n"/>
-      <c r="H36" s="86" t="n"/>
+      <c r="H36" s="77" t="n"/>
       <c r="I36" s="78" t="n"/>
     </row>
     <row r="37" ht="33" customHeight="1" s="47">
@@ -5023,9 +5563,9 @@
         </is>
       </c>
       <c r="E37" s="77" t="n"/>
-      <c r="F37" s="86" t="n"/>
+      <c r="F37" s="77" t="n"/>
       <c r="G37" s="77" t="n"/>
-      <c r="H37" s="86" t="n"/>
+      <c r="H37" s="77" t="n"/>
       <c r="I37" s="78" t="n"/>
     </row>
     <row r="38" ht="33" customHeight="1" s="47">
@@ -5042,9 +5582,9 @@
         </is>
       </c>
       <c r="E38" s="77" t="n"/>
-      <c r="F38" s="86" t="n"/>
+      <c r="F38" s="77" t="n"/>
       <c r="G38" s="77" t="n"/>
-      <c r="H38" s="86" t="n"/>
+      <c r="H38" s="77" t="n"/>
       <c r="I38" s="78" t="n"/>
     </row>
     <row r="39" ht="33" customHeight="1" s="47">
@@ -5061,9 +5601,9 @@
         </is>
       </c>
       <c r="E39" s="77" t="n"/>
-      <c r="F39" s="86" t="n"/>
+      <c r="F39" s="77" t="n"/>
       <c r="G39" s="77" t="n"/>
-      <c r="H39" s="86" t="n"/>
+      <c r="H39" s="77" t="n"/>
       <c r="I39" s="78" t="n"/>
     </row>
     <row r="40" ht="33" customHeight="1" s="47">
@@ -5080,9 +5620,9 @@
         </is>
       </c>
       <c r="E40" s="77" t="n"/>
-      <c r="F40" s="86" t="n"/>
+      <c r="F40" s="77" t="n"/>
       <c r="G40" s="77" t="n"/>
-      <c r="H40" s="86" t="n"/>
+      <c r="H40" s="77" t="n"/>
       <c r="I40" s="78" t="n"/>
     </row>
     <row r="41" ht="8" customHeight="1" s="47">
@@ -5104,11 +5644,11 @@
       </c>
       <c r="B42" s="77" t="n"/>
       <c r="C42" s="77" t="n"/>
-      <c r="D42" s="86" t="n"/>
+      <c r="D42" s="77" t="n"/>
       <c r="E42" s="77" t="n"/>
-      <c r="F42" s="86" t="n"/>
+      <c r="F42" s="77" t="n"/>
       <c r="G42" s="77" t="n"/>
-      <c r="H42" s="86" t="n"/>
+      <c r="H42" s="77" t="n"/>
       <c r="I42" s="78" t="n"/>
     </row>
   </sheetData>
@@ -5136,7 +5676,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5159,7 +5699,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕДНЕВНЫЙ ОТЧЁТ — ШАРКЕР  |  Данные из 1С</t>
         </is>
@@ -5173,8 +5713,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -5338,11 +5878,11 @@
       </c>
       <c r="B11" s="79" t="n"/>
       <c r="C11" s="79" t="n"/>
-      <c r="D11" s="84" t="n"/>
+      <c r="D11" s="79" t="n"/>
       <c r="E11" s="79" t="n"/>
-      <c r="F11" s="84" t="n"/>
+      <c r="F11" s="79" t="n"/>
       <c r="G11" s="79" t="n"/>
-      <c r="H11" s="84" t="n"/>
+      <c r="H11" s="79" t="n"/>
       <c r="I11" s="80" t="n"/>
     </row>
     <row r="12" ht="33" customHeight="1" s="47">
@@ -5359,7 +5899,7 @@
         </is>
       </c>
       <c r="E12" s="77" t="n"/>
-      <c r="F12" s="85" t="n"/>
+      <c r="F12" s="78" t="n"/>
       <c r="G12" s="68" t="n"/>
       <c r="H12" s="68" t="inlineStr">
         <is>
@@ -5378,7 +5918,7 @@
       <c r="C13" s="70" t="n"/>
       <c r="D13" s="81" t="n"/>
       <c r="E13" s="77" t="n"/>
-      <c r="F13" s="85" t="n"/>
+      <c r="F13" s="78" t="n"/>
       <c r="G13" s="70" t="n"/>
       <c r="H13" s="81" t="n"/>
       <c r="I13" s="78" t="n"/>
@@ -5393,7 +5933,7 @@
       <c r="C14" s="70" t="n"/>
       <c r="D14" s="81" t="n"/>
       <c r="E14" s="77" t="n"/>
-      <c r="F14" s="85" t="n"/>
+      <c r="F14" s="78" t="n"/>
       <c r="G14" s="70" t="n"/>
       <c r="H14" s="81" t="n"/>
       <c r="I14" s="78" t="n"/>
@@ -5408,7 +5948,7 @@
       <c r="C15" s="70" t="n"/>
       <c r="D15" s="81" t="n"/>
       <c r="E15" s="77" t="n"/>
-      <c r="F15" s="85" t="n"/>
+      <c r="F15" s="78" t="n"/>
       <c r="G15" s="70" t="n"/>
       <c r="H15" s="70" t="inlineStr">
         <is>
@@ -5427,7 +5967,7 @@
       <c r="C16" s="70" t="n"/>
       <c r="D16" s="81" t="n"/>
       <c r="E16" s="77" t="n"/>
-      <c r="F16" s="85" t="n"/>
+      <c r="F16" s="78" t="n"/>
       <c r="G16" s="70" t="n"/>
       <c r="H16" s="70" t="inlineStr">
         <is>
@@ -5446,7 +5986,7 @@
       <c r="C17" s="70" t="n"/>
       <c r="D17" s="81" t="n"/>
       <c r="E17" s="77" t="n"/>
-      <c r="F17" s="85" t="n"/>
+      <c r="F17" s="78" t="n"/>
       <c r="G17" s="70" t="n"/>
       <c r="H17" s="81" t="n"/>
       <c r="I17" s="78" t="n"/>
@@ -5470,11 +6010,11 @@
       </c>
       <c r="B19" s="79" t="n"/>
       <c r="C19" s="79" t="n"/>
-      <c r="D19" s="84" t="n"/>
+      <c r="D19" s="79" t="n"/>
       <c r="E19" s="79" t="n"/>
-      <c r="F19" s="84" t="n"/>
+      <c r="F19" s="79" t="n"/>
       <c r="G19" s="79" t="n"/>
-      <c r="H19" s="84" t="n"/>
+      <c r="H19" s="79" t="n"/>
       <c r="I19" s="80" t="n"/>
     </row>
     <row r="20" ht="33" customHeight="1" s="47">
@@ -5552,7 +6092,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="33" customHeight="1" s="47">
+    <row r="23" hidden="1" ht="33" customHeight="1" s="47">
       <c r="A23" s="69" t="n"/>
       <c r="B23" s="69" t="inlineStr">
         <is>
@@ -5574,7 +6114,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="48" customHeight="1" s="47">
+    <row r="24" hidden="1" ht="48" customHeight="1" s="47">
       <c r="A24" s="69" t="n"/>
       <c r="B24" s="69" t="inlineStr">
         <is>
@@ -5598,7 +6138,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1" s="47">
+    <row r="25" hidden="1" ht="48" customHeight="1" s="47">
       <c r="A25" s="69" t="n"/>
       <c r="B25" s="69" t="inlineStr">
         <is>
@@ -5641,11 +6181,11 @@
       </c>
       <c r="B27" s="77" t="n"/>
       <c r="C27" s="77" t="n"/>
-      <c r="D27" s="86" t="n"/>
+      <c r="D27" s="77" t="n"/>
       <c r="E27" s="77" t="n"/>
-      <c r="F27" s="86" t="n"/>
+      <c r="F27" s="77" t="n"/>
       <c r="G27" s="77" t="n"/>
-      <c r="H27" s="86" t="n"/>
+      <c r="H27" s="77" t="n"/>
       <c r="I27" s="78" t="n"/>
     </row>
   </sheetData>
@@ -5676,7 +6216,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5699,7 +6239,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — ШАРКЕР  |  Длинные ремонты</t>
         </is>
@@ -5713,8 +6253,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -5893,11 +6433,11 @@
       </c>
       <c r="B12" s="79" t="n"/>
       <c r="C12" s="79" t="n"/>
-      <c r="D12" s="84" t="n"/>
+      <c r="D12" s="79" t="n"/>
       <c r="E12" s="79" t="n"/>
-      <c r="F12" s="84" t="n"/>
+      <c r="F12" s="79" t="n"/>
       <c r="G12" s="79" t="n"/>
-      <c r="H12" s="84" t="n"/>
+      <c r="H12" s="79" t="n"/>
       <c r="I12" s="80" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1" s="47">
@@ -5914,7 +6454,7 @@
         </is>
       </c>
       <c r="E13" s="77" t="n"/>
-      <c r="F13" s="85" t="n"/>
+      <c r="F13" s="78" t="n"/>
       <c r="G13" s="68" t="n"/>
       <c r="H13" s="68" t="inlineStr">
         <is>
@@ -5933,7 +6473,7 @@
       <c r="C14" s="70" t="n"/>
       <c r="D14" s="81" t="n"/>
       <c r="E14" s="77" t="n"/>
-      <c r="F14" s="85" t="n"/>
+      <c r="F14" s="78" t="n"/>
       <c r="G14" s="70" t="n"/>
       <c r="H14" s="81" t="n"/>
       <c r="I14" s="78" t="n"/>
@@ -5948,7 +6488,7 @@
       <c r="C15" s="70" t="n"/>
       <c r="D15" s="81" t="n"/>
       <c r="E15" s="77" t="n"/>
-      <c r="F15" s="85" t="n"/>
+      <c r="F15" s="78" t="n"/>
       <c r="G15" s="70" t="n"/>
       <c r="H15" s="81" t="n"/>
       <c r="I15" s="78" t="n"/>
@@ -5963,7 +6503,7 @@
       <c r="C16" s="70" t="n"/>
       <c r="D16" s="81" t="n"/>
       <c r="E16" s="77" t="n"/>
-      <c r="F16" s="85" t="n"/>
+      <c r="F16" s="78" t="n"/>
       <c r="G16" s="70" t="n"/>
       <c r="H16" s="81" t="n"/>
       <c r="I16" s="78" t="n"/>
@@ -5978,7 +6518,7 @@
       <c r="C17" s="70" t="n"/>
       <c r="D17" s="82" t="n"/>
       <c r="E17" s="77" t="n"/>
-      <c r="F17" s="87" t="n"/>
+      <c r="F17" s="78" t="n"/>
       <c r="G17" s="70" t="n"/>
       <c r="H17" s="81" t="n"/>
       <c r="I17" s="78" t="n"/>
@@ -5993,7 +6533,7 @@
       <c r="C18" s="70" t="n"/>
       <c r="D18" s="81" t="n"/>
       <c r="E18" s="77" t="n"/>
-      <c r="F18" s="85" t="n"/>
+      <c r="F18" s="78" t="n"/>
       <c r="G18" s="70" t="n"/>
       <c r="H18" s="81" t="n"/>
       <c r="I18" s="78" t="n"/>
@@ -6008,7 +6548,7 @@
       <c r="C19" s="70" t="n"/>
       <c r="D19" s="81" t="n"/>
       <c r="E19" s="77" t="n"/>
-      <c r="F19" s="85" t="n"/>
+      <c r="F19" s="78" t="n"/>
       <c r="G19" s="70" t="n"/>
       <c r="H19" s="81" t="n"/>
       <c r="I19" s="78" t="n"/>
@@ -6023,7 +6563,7 @@
       <c r="C20" s="70" t="n"/>
       <c r="D20" s="81" t="n"/>
       <c r="E20" s="77" t="n"/>
-      <c r="F20" s="85" t="n"/>
+      <c r="F20" s="78" t="n"/>
       <c r="G20" s="70" t="n"/>
       <c r="H20" s="81" t="n"/>
       <c r="I20" s="78" t="n"/>
@@ -6038,7 +6578,7 @@
       <c r="C21" s="70" t="n"/>
       <c r="D21" s="81" t="n"/>
       <c r="E21" s="77" t="n"/>
-      <c r="F21" s="85" t="n"/>
+      <c r="F21" s="78" t="n"/>
       <c r="G21" s="70" t="n"/>
       <c r="H21" s="81" t="n"/>
       <c r="I21" s="78" t="n"/>
@@ -6053,7 +6593,7 @@
       <c r="C22" s="70" t="n"/>
       <c r="D22" s="81" t="n"/>
       <c r="E22" s="77" t="n"/>
-      <c r="F22" s="85" t="n"/>
+      <c r="F22" s="78" t="n"/>
       <c r="G22" s="70" t="n"/>
       <c r="H22" s="81" t="n"/>
       <c r="I22" s="78" t="n"/>
@@ -6068,7 +6608,7 @@
       <c r="C23" s="70" t="n"/>
       <c r="D23" s="81" t="n"/>
       <c r="E23" s="77" t="n"/>
-      <c r="F23" s="85" t="n"/>
+      <c r="F23" s="78" t="n"/>
       <c r="G23" s="70" t="n"/>
       <c r="H23" s="81" t="n"/>
       <c r="I23" s="78" t="n"/>
@@ -6092,11 +6632,11 @@
       </c>
       <c r="B25" s="79" t="n"/>
       <c r="C25" s="79" t="n"/>
-      <c r="D25" s="84" t="n"/>
+      <c r="D25" s="79" t="n"/>
       <c r="E25" s="79" t="n"/>
-      <c r="F25" s="84" t="n"/>
+      <c r="F25" s="79" t="n"/>
       <c r="G25" s="79" t="n"/>
-      <c r="H25" s="84" t="n"/>
+      <c r="H25" s="79" t="n"/>
       <c r="I25" s="80" t="n"/>
     </row>
     <row r="26" ht="33" customHeight="1" s="47">
@@ -6297,11 +6837,11 @@
       </c>
       <c r="B36" s="79" t="n"/>
       <c r="C36" s="79" t="n"/>
-      <c r="D36" s="84" t="n"/>
+      <c r="D36" s="79" t="n"/>
       <c r="E36" s="79" t="n"/>
-      <c r="F36" s="84" t="n"/>
+      <c r="F36" s="79" t="n"/>
       <c r="G36" s="79" t="n"/>
-      <c r="H36" s="84" t="n"/>
+      <c r="H36" s="79" t="n"/>
       <c r="I36" s="80" t="n"/>
     </row>
     <row r="37" ht="33" customHeight="1" s="47">
@@ -6318,9 +6858,9 @@
         </is>
       </c>
       <c r="E37" s="77" t="n"/>
-      <c r="F37" s="86" t="n"/>
+      <c r="F37" s="77" t="n"/>
       <c r="G37" s="77" t="n"/>
-      <c r="H37" s="86" t="n"/>
+      <c r="H37" s="77" t="n"/>
       <c r="I37" s="78" t="n"/>
     </row>
     <row r="38" ht="33" customHeight="1" s="47">
@@ -6337,9 +6877,9 @@
         </is>
       </c>
       <c r="E38" s="77" t="n"/>
-      <c r="F38" s="86" t="n"/>
+      <c r="F38" s="77" t="n"/>
       <c r="G38" s="77" t="n"/>
-      <c r="H38" s="86" t="n"/>
+      <c r="H38" s="77" t="n"/>
       <c r="I38" s="78" t="n"/>
     </row>
     <row r="39" ht="33" customHeight="1" s="47">
@@ -6356,9 +6896,9 @@
         </is>
       </c>
       <c r="E39" s="77" t="n"/>
-      <c r="F39" s="86" t="n"/>
+      <c r="F39" s="77" t="n"/>
       <c r="G39" s="77" t="n"/>
-      <c r="H39" s="86" t="n"/>
+      <c r="H39" s="77" t="n"/>
       <c r="I39" s="78" t="n"/>
     </row>
     <row r="40" ht="8" customHeight="1" s="47">
@@ -6380,11 +6920,11 @@
       </c>
       <c r="B41" s="77" t="n"/>
       <c r="C41" s="77" t="n"/>
-      <c r="D41" s="86" t="n"/>
+      <c r="D41" s="77" t="n"/>
       <c r="E41" s="77" t="n"/>
-      <c r="F41" s="86" t="n"/>
+      <c r="F41" s="77" t="n"/>
       <c r="G41" s="77" t="n"/>
-      <c r="H41" s="86" t="n"/>
+      <c r="H41" s="77" t="n"/>
       <c r="I41" s="78" t="n"/>
     </row>
   </sheetData>
@@ -6430,7 +6970,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6453,7 +6993,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕДНЕВНЫЙ ОТЧЁТ — ЦКР  |  Данные из 1С</t>
         </is>
@@ -6467,8 +7007,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -6613,7 +7153,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="33" customHeight="1" s="47">
+    <row r="10" hidden="1" ht="33" customHeight="1" s="47">
       <c r="A10" s="69" t="n"/>
       <c r="B10" s="69" t="inlineStr">
         <is>
@@ -6654,11 +7194,11 @@
       </c>
       <c r="B12" s="79" t="n"/>
       <c r="C12" s="79" t="n"/>
-      <c r="D12" s="84" t="n"/>
+      <c r="D12" s="79" t="n"/>
       <c r="E12" s="79" t="n"/>
-      <c r="F12" s="84" t="n"/>
+      <c r="F12" s="79" t="n"/>
       <c r="G12" s="79" t="n"/>
-      <c r="H12" s="84" t="n"/>
+      <c r="H12" s="79" t="n"/>
       <c r="I12" s="80" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1" s="47">
@@ -6675,13 +7215,9 @@
         </is>
       </c>
       <c r="E13" s="77" t="n"/>
-      <c r="F13" s="85" t="n"/>
+      <c r="F13" s="78" t="n"/>
       <c r="G13" s="68" t="n"/>
-      <c r="H13" s="68" t="inlineStr">
-        <is>
-          <t>Норма</t>
-        </is>
-      </c>
+      <c r="H13" s="92" t="n"/>
       <c r="I13" s="78" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
@@ -6694,9 +7230,9 @@
       <c r="C14" s="70" t="n"/>
       <c r="D14" s="81" t="n"/>
       <c r="E14" s="77" t="n"/>
-      <c r="F14" s="85" t="n"/>
+      <c r="F14" s="78" t="n"/>
       <c r="G14" s="70" t="n"/>
-      <c r="H14" s="81" t="n"/>
+      <c r="H14" s="93" t="n"/>
       <c r="I14" s="78" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1" s="47">
@@ -6709,9 +7245,9 @@
       <c r="C15" s="70" t="n"/>
       <c r="D15" s="81" t="n"/>
       <c r="E15" s="77" t="n"/>
-      <c r="F15" s="85" t="n"/>
+      <c r="F15" s="78" t="n"/>
       <c r="G15" s="70" t="n"/>
-      <c r="H15" s="81" t="n"/>
+      <c r="H15" s="93" t="n"/>
       <c r="I15" s="78" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1" s="47">
@@ -6724,13 +7260,9 @@
       <c r="C16" s="70" t="n"/>
       <c r="D16" s="81" t="n"/>
       <c r="E16" s="77" t="n"/>
-      <c r="F16" s="85" t="n"/>
+      <c r="F16" s="78" t="n"/>
       <c r="G16" s="70" t="n"/>
-      <c r="H16" s="70" t="inlineStr">
-        <is>
-          <t>Цель: 0</t>
-        </is>
-      </c>
+      <c r="H16" s="94" t="n"/>
       <c r="I16" s="78" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1" s="47">
@@ -6743,13 +7275,9 @@
       <c r="C17" s="70" t="n"/>
       <c r="D17" s="81" t="n"/>
       <c r="E17" s="77" t="n"/>
-      <c r="F17" s="85" t="n"/>
+      <c r="F17" s="78" t="n"/>
       <c r="G17" s="70" t="n"/>
-      <c r="H17" s="70" t="inlineStr">
-        <is>
-          <t>Цель: 0</t>
-        </is>
-      </c>
+      <c r="H17" s="94" t="n"/>
       <c r="I17" s="78" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1" s="47">
@@ -6762,9 +7290,9 @@
       <c r="C18" s="70" t="n"/>
       <c r="D18" s="81" t="n"/>
       <c r="E18" s="77" t="n"/>
-      <c r="F18" s="85" t="n"/>
+      <c r="F18" s="78" t="n"/>
       <c r="G18" s="70" t="n"/>
-      <c r="H18" s="81" t="n"/>
+      <c r="H18" s="93" t="n"/>
       <c r="I18" s="78" t="n"/>
     </row>
     <row r="19" ht="8" customHeight="1" s="47">
@@ -6775,8 +7303,8 @@
       <c r="E19" s="55" t="n"/>
       <c r="F19" s="83" t="n"/>
       <c r="G19" s="55" t="n"/>
-      <c r="H19" s="83" t="n"/>
-      <c r="I19" s="55" t="n"/>
+      <c r="H19" s="95" t="n"/>
+      <c r="I19" s="96" t="n"/>
     </row>
     <row r="20" ht="33" customHeight="1" s="47">
       <c r="A20" s="67" t="inlineStr">
@@ -6786,11 +7314,11 @@
       </c>
       <c r="B20" s="79" t="n"/>
       <c r="C20" s="79" t="n"/>
-      <c r="D20" s="84" t="n"/>
+      <c r="D20" s="79" t="n"/>
       <c r="E20" s="79" t="n"/>
-      <c r="F20" s="84" t="n"/>
+      <c r="F20" s="79" t="n"/>
       <c r="G20" s="79" t="n"/>
-      <c r="H20" s="84" t="n"/>
+      <c r="H20" s="79" t="n"/>
       <c r="I20" s="80" t="n"/>
     </row>
     <row r="21" ht="33" customHeight="1" s="47">
@@ -6868,7 +7396,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="33" customHeight="1" s="47">
+    <row r="24" hidden="1" ht="33" customHeight="1" s="47">
       <c r="A24" s="69" t="n"/>
       <c r="B24" s="69" t="inlineStr">
         <is>
@@ -6890,7 +7418,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="48" customHeight="1" s="47">
+    <row r="25" hidden="1" ht="48" customHeight="1" s="47">
       <c r="A25" s="69" t="n"/>
       <c r="B25" s="69" t="inlineStr">
         <is>
@@ -6914,7 +7442,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="48" customHeight="1" s="47">
+    <row r="26" hidden="1" ht="48" customHeight="1" s="47">
       <c r="A26" s="69" t="n"/>
       <c r="B26" s="69" t="inlineStr">
         <is>
@@ -6957,11 +7485,11 @@
       </c>
       <c r="B28" s="77" t="n"/>
       <c r="C28" s="77" t="n"/>
-      <c r="D28" s="86" t="n"/>
+      <c r="D28" s="77" t="n"/>
       <c r="E28" s="77" t="n"/>
-      <c r="F28" s="86" t="n"/>
+      <c r="F28" s="77" t="n"/>
       <c r="G28" s="77" t="n"/>
-      <c r="H28" s="86" t="n"/>
+      <c r="H28" s="77" t="n"/>
       <c r="I28" s="78" t="n"/>
     </row>
   </sheetData>
@@ -6992,7 +7520,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7015,7 +7543,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
+      <c r="A1" s="90" t="inlineStr">
         <is>
           <t>ЕЖЕНЕДЕЛЬНЫЙ ОТЧЁТ — ЦКР  |  Длинные ремонты</t>
         </is>
@@ -7029,8 +7557,8 @@
       <c r="H1" s="75" t="n"/>
       <c r="I1" s="75" t="n"/>
     </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
+    <row r="2" hidden="1" ht="32" customHeight="1" s="47">
+      <c r="A2" s="91" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
         </is>
@@ -7209,11 +7737,11 @@
       </c>
       <c r="B12" s="79" t="n"/>
       <c r="C12" s="79" t="n"/>
-      <c r="D12" s="84" t="n"/>
+      <c r="D12" s="79" t="n"/>
       <c r="E12" s="79" t="n"/>
-      <c r="F12" s="84" t="n"/>
+      <c r="F12" s="79" t="n"/>
       <c r="G12" s="79" t="n"/>
-      <c r="H12" s="84" t="n"/>
+      <c r="H12" s="79" t="n"/>
       <c r="I12" s="80" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1" s="47">
@@ -7230,13 +7758,9 @@
         </is>
       </c>
       <c r="E13" s="77" t="n"/>
-      <c r="F13" s="85" t="n"/>
+      <c r="F13" s="78" t="n"/>
       <c r="G13" s="68" t="n"/>
-      <c r="H13" s="68" t="inlineStr">
-        <is>
-          <t>vs пред. нед.</t>
-        </is>
-      </c>
+      <c r="H13" s="92" t="n"/>
       <c r="I13" s="78" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
@@ -7249,9 +7773,9 @@
       <c r="C14" s="70" t="n"/>
       <c r="D14" s="81" t="n"/>
       <c r="E14" s="77" t="n"/>
-      <c r="F14" s="85" t="n"/>
+      <c r="F14" s="78" t="n"/>
       <c r="G14" s="70" t="n"/>
-      <c r="H14" s="81" t="n"/>
+      <c r="H14" s="93" t="n"/>
       <c r="I14" s="78" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1" s="47">
@@ -7264,9 +7788,9 @@
       <c r="C15" s="70" t="n"/>
       <c r="D15" s="81" t="n"/>
       <c r="E15" s="77" t="n"/>
-      <c r="F15" s="85" t="n"/>
+      <c r="F15" s="78" t="n"/>
       <c r="G15" s="70" t="n"/>
-      <c r="H15" s="81" t="n"/>
+      <c r="H15" s="93" t="n"/>
       <c r="I15" s="78" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1" s="47">
@@ -7279,9 +7803,9 @@
       <c r="C16" s="70" t="n"/>
       <c r="D16" s="81" t="n"/>
       <c r="E16" s="77" t="n"/>
-      <c r="F16" s="85" t="n"/>
+      <c r="F16" s="78" t="n"/>
       <c r="G16" s="70" t="n"/>
-      <c r="H16" s="81" t="n"/>
+      <c r="H16" s="93" t="n"/>
       <c r="I16" s="78" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1" s="47">
@@ -7294,9 +7818,9 @@
       <c r="C17" s="70" t="n"/>
       <c r="D17" s="82" t="n"/>
       <c r="E17" s="77" t="n"/>
-      <c r="F17" s="87" t="n"/>
+      <c r="F17" s="78" t="n"/>
       <c r="G17" s="70" t="n"/>
-      <c r="H17" s="81" t="n"/>
+      <c r="H17" s="93" t="n"/>
       <c r="I17" s="78" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1" s="47">
@@ -7309,9 +7833,9 @@
       <c r="C18" s="70" t="n"/>
       <c r="D18" s="81" t="n"/>
       <c r="E18" s="77" t="n"/>
-      <c r="F18" s="85" t="n"/>
+      <c r="F18" s="78" t="n"/>
       <c r="G18" s="70" t="n"/>
-      <c r="H18" s="81" t="n"/>
+      <c r="H18" s="93" t="n"/>
       <c r="I18" s="78" t="n"/>
     </row>
     <row r="19" ht="33" customHeight="1" s="47">
@@ -7324,9 +7848,9 @@
       <c r="C19" s="70" t="n"/>
       <c r="D19" s="81" t="n"/>
       <c r="E19" s="77" t="n"/>
-      <c r="F19" s="85" t="n"/>
+      <c r="F19" s="78" t="n"/>
       <c r="G19" s="70" t="n"/>
-      <c r="H19" s="81" t="n"/>
+      <c r="H19" s="93" t="n"/>
       <c r="I19" s="78" t="n"/>
     </row>
     <row r="20" ht="33" customHeight="1" s="47">
@@ -7339,9 +7863,9 @@
       <c r="C20" s="70" t="n"/>
       <c r="D20" s="81" t="n"/>
       <c r="E20" s="77" t="n"/>
-      <c r="F20" s="85" t="n"/>
+      <c r="F20" s="78" t="n"/>
       <c r="G20" s="70" t="n"/>
-      <c r="H20" s="81" t="n"/>
+      <c r="H20" s="93" t="n"/>
       <c r="I20" s="78" t="n"/>
     </row>
     <row r="21" ht="33" customHeight="1" s="47">
@@ -7354,9 +7878,9 @@
       <c r="C21" s="70" t="n"/>
       <c r="D21" s="81" t="n"/>
       <c r="E21" s="77" t="n"/>
-      <c r="F21" s="85" t="n"/>
+      <c r="F21" s="78" t="n"/>
       <c r="G21" s="70" t="n"/>
-      <c r="H21" s="81" t="n"/>
+      <c r="H21" s="93" t="n"/>
       <c r="I21" s="78" t="n"/>
     </row>
     <row r="22" ht="8" customHeight="1" s="47">
@@ -7378,11 +7902,11 @@
       </c>
       <c r="B23" s="79" t="n"/>
       <c r="C23" s="79" t="n"/>
-      <c r="D23" s="84" t="n"/>
+      <c r="D23" s="79" t="n"/>
       <c r="E23" s="79" t="n"/>
-      <c r="F23" s="84" t="n"/>
+      <c r="F23" s="79" t="n"/>
       <c r="G23" s="79" t="n"/>
-      <c r="H23" s="84" t="n"/>
+      <c r="H23" s="79" t="n"/>
       <c r="I23" s="80" t="n"/>
     </row>
     <row r="24" ht="33" customHeight="1" s="47">
@@ -7582,11 +8106,11 @@
       </c>
       <c r="B34" s="79" t="n"/>
       <c r="C34" s="79" t="n"/>
-      <c r="D34" s="84" t="n"/>
+      <c r="D34" s="79" t="n"/>
       <c r="E34" s="79" t="n"/>
-      <c r="F34" s="84" t="n"/>
+      <c r="F34" s="79" t="n"/>
       <c r="G34" s="79" t="n"/>
-      <c r="H34" s="84" t="n"/>
+      <c r="H34" s="79" t="n"/>
       <c r="I34" s="80" t="n"/>
     </row>
     <row r="35" ht="33" customHeight="1" s="47">
@@ -7603,9 +8127,9 @@
         </is>
       </c>
       <c r="E35" s="77" t="n"/>
-      <c r="F35" s="86" t="n"/>
+      <c r="F35" s="77" t="n"/>
       <c r="G35" s="77" t="n"/>
-      <c r="H35" s="86" t="n"/>
+      <c r="H35" s="77" t="n"/>
       <c r="I35" s="78" t="n"/>
     </row>
     <row r="36" ht="33" customHeight="1" s="47">
@@ -7622,9 +8146,9 @@
         </is>
       </c>
       <c r="E36" s="77" t="n"/>
-      <c r="F36" s="86" t="n"/>
+      <c r="F36" s="77" t="n"/>
       <c r="G36" s="77" t="n"/>
-      <c r="H36" s="86" t="n"/>
+      <c r="H36" s="77" t="n"/>
       <c r="I36" s="78" t="n"/>
     </row>
     <row r="37" ht="33" customHeight="1" s="47">
@@ -7641,9 +8165,9 @@
         </is>
       </c>
       <c r="E37" s="77" t="n"/>
-      <c r="F37" s="86" t="n"/>
+      <c r="F37" s="77" t="n"/>
       <c r="G37" s="77" t="n"/>
-      <c r="H37" s="86" t="n"/>
+      <c r="H37" s="77" t="n"/>
       <c r="I37" s="78" t="n"/>
     </row>
     <row r="38" ht="8" customHeight="1" s="47">
@@ -7665,11 +8189,11 @@
       </c>
       <c r="B39" s="77" t="n"/>
       <c r="C39" s="77" t="n"/>
-      <c r="D39" s="86" t="n"/>
+      <c r="D39" s="77" t="n"/>
       <c r="E39" s="77" t="n"/>
-      <c r="F39" s="86" t="n"/>
+      <c r="F39" s="77" t="n"/>
       <c r="G39" s="77" t="n"/>
-      <c r="H39" s="86" t="n"/>
+      <c r="H39" s="77" t="n"/>
       <c r="I39" s="78" t="n"/>
     </row>
   </sheetData>
@@ -7709,374 +8233,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:I17"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col width="2" customWidth="1" style="47" min="1" max="1"/>
-    <col width="48" customWidth="1" style="47" min="2" max="2"/>
-    <col width="2" customWidth="1" style="47" min="3" max="3"/>
-    <col width="15" customWidth="1" style="47" min="4" max="4"/>
-    <col width="2" customWidth="1" style="47" min="5" max="5"/>
-    <col width="15" customWidth="1" style="47" min="6" max="6"/>
-    <col width="2" customWidth="1" style="47" min="7" max="7"/>
-    <col width="14" customWidth="1" style="47" min="8" max="8"/>
-    <col width="16" customWidth="1" style="47" min="9" max="9"/>
-    <col hidden="1" width="2" customWidth="1" style="47" min="10" max="10"/>
-    <col hidden="1" width="2" customWidth="1" style="47" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="34" customHeight="1" s="47">
-      <c r="A1" s="62" t="inlineStr">
-        <is>
-          <t>ЕЖЕДНЕВНЫЙ ОТЧЁТ — МОЙКА  |  Данные из 1С</t>
-        </is>
-      </c>
-      <c r="B1" s="75" t="n"/>
-      <c r="C1" s="75" t="n"/>
-      <c r="D1" s="75" t="n"/>
-      <c r="E1" s="75" t="n"/>
-      <c r="F1" s="75" t="n"/>
-      <c r="G1" s="75" t="n"/>
-      <c r="H1" s="75" t="n"/>
-      <c r="I1" s="75" t="n"/>
-    </row>
-    <row r="2" ht="32" customHeight="1" s="47">
-      <c r="A2" s="63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  🔵 Синий = из 1С автоматически     🟡 Жёлтый = вводит руководитель</t>
-        </is>
-      </c>
-      <c r="B2" s="76" t="n"/>
-      <c r="C2" s="76" t="n"/>
-      <c r="D2" s="76" t="n"/>
-      <c r="E2" s="76" t="n"/>
-      <c r="F2" s="76" t="n"/>
-      <c r="G2" s="76" t="n"/>
-      <c r="H2" s="76" t="n"/>
-      <c r="I2" s="76" t="n"/>
-    </row>
-    <row r="3" ht="30" customHeight="1" s="47">
-      <c r="A3" s="64" t="n"/>
-      <c r="B3" s="65" t="inlineStr">
-        <is>
-          <t>АТЦ:</t>
-        </is>
-      </c>
-      <c r="C3" s="64" t="n"/>
-      <c r="D3" s="66" t="n"/>
-      <c r="E3" s="77" t="n"/>
-      <c r="F3" s="77" t="n"/>
-      <c r="G3" s="77" t="n"/>
-      <c r="H3" s="77" t="n"/>
-      <c r="I3" s="78" t="n"/>
-    </row>
-    <row r="4" ht="30" customHeight="1" s="47">
-      <c r="A4" s="64" t="n"/>
-      <c r="B4" s="65" t="inlineStr">
-        <is>
-          <t>Дата (авто):</t>
-        </is>
-      </c>
-      <c r="C4" s="64" t="n"/>
-      <c r="D4" s="66" t="n"/>
-      <c r="E4" s="77" t="n"/>
-      <c r="F4" s="77" t="n"/>
-      <c r="G4" s="77" t="n"/>
-      <c r="H4" s="77" t="n"/>
-      <c r="I4" s="78" t="n"/>
-    </row>
-    <row r="5" ht="26" customHeight="1" s="47">
-      <c r="A5" s="64" t="n"/>
-      <c r="B5" s="65" t="n"/>
-      <c r="C5" s="64" t="n"/>
-      <c r="D5" s="66" t="n"/>
-      <c r="E5" s="66" t="n"/>
-      <c r="F5" s="66" t="n"/>
-      <c r="G5" s="66" t="n"/>
-      <c r="H5" s="66" t="n"/>
-      <c r="I5" s="66" t="n"/>
-    </row>
-    <row r="6" ht="33" customHeight="1" s="47">
-      <c r="A6" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  КЛЮЧЕВЫЕ ПОКАЗАТЕЛИ (из 1С) Мойка на ул. Строителей</t>
-        </is>
-      </c>
-      <c r="B6" s="79" t="n"/>
-      <c r="C6" s="79" t="n"/>
-      <c r="D6" s="79" t="n"/>
-      <c r="E6" s="79" t="n"/>
-      <c r="F6" s="79" t="n"/>
-      <c r="G6" s="79" t="n"/>
-      <c r="H6" s="79" t="n"/>
-      <c r="I6" s="80" t="n"/>
-    </row>
-    <row r="7" ht="33" customHeight="1" s="47">
-      <c r="A7" s="68" t="n"/>
-      <c r="B7" s="68" t="inlineStr">
-        <is>
-          <t>Показатель</t>
-        </is>
-      </c>
-      <c r="C7" s="68" t="n"/>
-      <c r="D7" s="68" t="inlineStr">
-        <is>
-          <t>ПЛАН</t>
-        </is>
-      </c>
-      <c r="E7" s="68" t="n"/>
-      <c r="F7" s="68" t="inlineStr">
-        <is>
-          <t>ФАКТ (1С)</t>
-        </is>
-      </c>
-      <c r="G7" s="68" t="n"/>
-      <c r="H7" s="68" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="I7" s="68" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="33" customHeight="1" s="47">
-      <c r="A8" s="69" t="n"/>
-      <c r="B8" s="69" t="inlineStr">
-        <is>
-          <t>Машин обслужено</t>
-        </is>
-      </c>
-      <c r="C8" s="70" t="n"/>
-      <c r="D8" s="81" t="n"/>
-      <c r="E8" s="70" t="n"/>
-      <c r="F8" s="81" t="n"/>
-      <c r="G8" s="70" t="n"/>
-      <c r="H8" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D8),ISNUMBER(F8),D8&gt;0),F8/D8,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I8" s="70" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="33" customHeight="1" s="47">
-      <c r="A9" s="69" t="n"/>
-      <c r="B9" s="69" t="inlineStr">
-        <is>
-          <t>Выручка за день</t>
-        </is>
-      </c>
-      <c r="C9" s="70" t="n"/>
-      <c r="D9" s="81" t="n"/>
-      <c r="E9" s="70" t="n"/>
-      <c r="F9" s="81" t="n"/>
-      <c r="G9" s="70" t="n"/>
-      <c r="H9" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D9),ISNUMBER(F9),D9&gt;0),F9/D9,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I9" s="70" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="33" customHeight="1" s="47">
-      <c r="A10" s="69" t="n"/>
-      <c r="B10" s="69" t="inlineStr">
-        <is>
-          <t>Средний чек (руб./машина)</t>
-        </is>
-      </c>
-      <c r="C10" s="70" t="n"/>
-      <c r="D10" s="81">
-        <f>IFERROR(D9/D8,"—")</f>
-        <v/>
-      </c>
-      <c r="E10" s="70" t="n"/>
-      <c r="F10" s="81">
-        <f>IFERROR(F9/F8,"—")</f>
-        <v/>
-      </c>
-      <c r="G10" s="70" t="n"/>
-      <c r="H10" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D10),ISNUMBER(F10),D10&gt;0),F10/D10,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I10" s="70" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="8" customHeight="1" s="47">
-      <c r="A11" s="55" t="n"/>
-      <c r="B11" s="55" t="n"/>
-      <c r="C11" s="55" t="n"/>
-      <c r="D11" s="83" t="n"/>
-      <c r="E11" s="55" t="n"/>
-      <c r="F11" s="83" t="n"/>
-      <c r="G11" s="55" t="n"/>
-      <c r="H11" s="83" t="n"/>
-      <c r="I11" s="55" t="n"/>
-    </row>
-    <row r="12" ht="33" customHeight="1" s="47" thickBot="1">
-      <c r="A12" s="67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  КЛЮЧЕВЫЕ ПОКАЗАТЕЛИ (из 1С) Мойка на ул. Ульяновская</t>
-        </is>
-      </c>
-      <c r="B12" s="79" t="n"/>
-      <c r="C12" s="79" t="n"/>
-      <c r="D12" s="84" t="n"/>
-      <c r="E12" s="79" t="n"/>
-      <c r="F12" s="84" t="n"/>
-      <c r="G12" s="79" t="n"/>
-      <c r="H12" s="84" t="n"/>
-      <c r="I12" s="80" t="n"/>
-    </row>
-    <row r="13" ht="33" customHeight="1" s="47">
-      <c r="A13" s="68" t="n"/>
-      <c r="B13" s="68" t="inlineStr">
-        <is>
-          <t>Показатель</t>
-        </is>
-      </c>
-      <c r="C13" s="68" t="n"/>
-      <c r="D13" s="68" t="inlineStr">
-        <is>
-          <t>ПЛАН</t>
-        </is>
-      </c>
-      <c r="E13" s="68" t="n"/>
-      <c r="F13" s="68" t="inlineStr">
-        <is>
-          <t>ФАКТ (1С)</t>
-        </is>
-      </c>
-      <c r="G13" s="68" t="n"/>
-      <c r="H13" s="68" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="I13" s="68" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="33" customHeight="1" s="47">
-      <c r="A14" s="69" t="n"/>
-      <c r="B14" s="69" t="inlineStr">
-        <is>
-          <t>Машин обслужено</t>
-        </is>
-      </c>
-      <c r="C14" s="70" t="n"/>
-      <c r="D14" s="81" t="n"/>
-      <c r="E14" s="70" t="n"/>
-      <c r="F14" s="81" t="n"/>
-      <c r="G14" s="70" t="n"/>
-      <c r="H14" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D14),ISNUMBER(F14),D14&gt;0),F14/D14,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I14" s="70" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="33" customHeight="1" s="47">
-      <c r="A15" s="69" t="n"/>
-      <c r="B15" s="69" t="inlineStr">
-        <is>
-          <t>Выручка за день</t>
-        </is>
-      </c>
-      <c r="C15" s="70" t="n"/>
-      <c r="D15" s="81" t="n"/>
-      <c r="E15" s="70" t="n"/>
-      <c r="F15" s="81" t="n"/>
-      <c r="G15" s="70" t="n"/>
-      <c r="H15" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D15),ISNUMBER(F15),D15&gt;0),F15/D15,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I15" s="70" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="33" customHeight="1" s="47">
-      <c r="A16" s="69" t="n"/>
-      <c r="B16" s="69" t="inlineStr">
-        <is>
-          <t>Средний чек (руб./машина)</t>
-        </is>
-      </c>
-      <c r="C16" s="70" t="n"/>
-      <c r="D16" s="81">
-        <f>IFERROR(D15/D14,"—")</f>
-        <v/>
-      </c>
-      <c r="E16" s="70" t="n"/>
-      <c r="F16" s="81">
-        <f>IFERROR(F15/F14,"—")</f>
-        <v/>
-      </c>
-      <c r="G16" s="70" t="n"/>
-      <c r="H16" s="82">
-        <f>IFERROR(IF(AND(ISNUMBER(D16),ISNUMBER(F16),D16&gt;0),F16/D16,"—"),"—")</f>
-        <v/>
-      </c>
-      <c r="I16" s="70" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="33" customHeight="1" s="47">
-      <c r="A17" s="69" t="inlineStr">
-        <is>
-          <t>🤖 Генерируется автоматически в 11:00 | Данные: 1С Альфа-Авто | Отправка: Битрикс24</t>
-        </is>
-      </c>
-      <c r="B17" s="77" t="n"/>
-      <c r="C17" s="77" t="n"/>
-      <c r="D17" s="86" t="n"/>
-      <c r="E17" s="77" t="n"/>
-      <c r="F17" s="86" t="n"/>
-      <c r="G17" s="77" t="n"/>
-      <c r="H17" s="86" t="n"/>
-      <c r="I17" s="78" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="D4:I4"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A17:I17"/>
-    <mergeCell ref="A6:I6"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="A12:I12"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Update shop weekly report comparisons
</commit_message>
<xml_diff>
--- a/backend/templates/report_template.xlsx
+++ b/backend/templates/report_template.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="713" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="СПРАВОЧНИК РУКОВОДИТЕЛЕЙ" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet name="Арсенал (Д)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Арсенал (Н)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Реф.сервис (Д)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Реф.сервис (Н)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Шаркер (Д)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Шаркер (Н)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ЦКР (Д)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ЦКР (Н)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Мойка (Д)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Мойка ул. Строителей (Н)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Мойка Ульяновская (Н)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="СПРАВОЧНИК РУКОВОДИТЕЛЕЙ" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Арсенал (Д)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Арсенал (Н)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реф.сервис (Д)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Реф.сервис (Н)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Шаркер (Д)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Шаркер (Н)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ЦКР (Д)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ЦКР (Н)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мойка (Д)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мойка ул. Строителей (Н)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Мойка Ульяновская (Н)" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Арсенал (Д)'!$A$1:$I$26</definedName>
@@ -709,7 +709,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -958,6 +958,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="24" fillId="19" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1398,7 +1401,11 @@
     </row>
     <row r="5" ht="26" customHeight="1" s="47">
       <c r="A5" s="64" t="n"/>
-      <c r="B5" s="65" t="n"/>
+      <c r="B5" s="65" t="inlineStr">
+        <is>
+          <t>Руководитель (авто):</t>
+        </is>
+      </c>
       <c r="C5" s="64" t="n"/>
       <c r="D5" s="66" t="n"/>
       <c r="E5" s="66" t="n"/>
@@ -2972,7 +2979,11 @@
     </row>
     <row r="5" ht="26" customHeight="1" s="47">
       <c r="A5" s="64" t="n"/>
-      <c r="B5" s="65" t="n"/>
+      <c r="B5" s="65" t="inlineStr">
+        <is>
+          <t>Руководитель (авто):</t>
+        </is>
+      </c>
       <c r="C5" s="64" t="n"/>
       <c r="D5" s="66" t="n"/>
       <c r="E5" s="66" t="n"/>
@@ -4366,7 +4377,11 @@
     </row>
     <row r="5" ht="26" customHeight="1" s="47">
       <c r="A5" s="64" t="n"/>
-      <c r="B5" s="65" t="n"/>
+      <c r="B5" s="65" t="inlineStr">
+        <is>
+          <t>Руководитель (авто):</t>
+        </is>
+      </c>
       <c r="C5" s="64" t="n"/>
       <c r="D5" s="66" t="n"/>
       <c r="E5" s="66" t="n"/>
@@ -5760,7 +5775,11 @@
     </row>
     <row r="5" ht="26" customHeight="1" s="47">
       <c r="A5" s="64" t="n"/>
-      <c r="B5" s="65" t="n"/>
+      <c r="B5" s="65" t="inlineStr">
+        <is>
+          <t>Руководитель (авто):</t>
+        </is>
+      </c>
       <c r="C5" s="64" t="n"/>
       <c r="D5" s="66" t="n"/>
       <c r="E5" s="66" t="n"/>
@@ -6232,8 +6251,8 @@
     <col width="2" customWidth="1" style="47" min="5" max="5"/>
     <col width="15" customWidth="1" style="47" min="6" max="6"/>
     <col width="2" customWidth="1" style="47" min="7" max="7"/>
-    <col width="14" customWidth="1" style="47" min="8" max="8"/>
-    <col width="16" customWidth="1" style="47" min="9" max="9"/>
+    <col width="15" customWidth="1" style="47" min="8" max="8"/>
+    <col width="12" customWidth="1" style="47" min="9" max="9"/>
     <col hidden="1" width="2" customWidth="1" style="47" min="10" max="10"/>
     <col hidden="1" width="2" customWidth="1" style="47" min="11" max="11"/>
   </cols>
@@ -6461,7 +6480,11 @@
           <t>vs пред. нед.</t>
         </is>
       </c>
-      <c r="I13" s="78" t="n"/>
+      <c r="I13" s="97" t="inlineStr">
+        <is>
+          <t>Δ %</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
       <c r="A14" s="69" t="n"/>
@@ -6476,7 +6499,7 @@
       <c r="F14" s="78" t="n"/>
       <c r="G14" s="70" t="n"/>
       <c r="H14" s="81" t="n"/>
-      <c r="I14" s="78" t="n"/>
+      <c r="I14" s="82" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1" s="47">
       <c r="A15" s="69" t="n"/>
@@ -6491,7 +6514,7 @@
       <c r="F15" s="78" t="n"/>
       <c r="G15" s="70" t="n"/>
       <c r="H15" s="81" t="n"/>
-      <c r="I15" s="78" t="n"/>
+      <c r="I15" s="82" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1" s="47">
       <c r="A16" s="69" t="n"/>
@@ -6506,13 +6529,13 @@
       <c r="F16" s="78" t="n"/>
       <c r="G16" s="70" t="n"/>
       <c r="H16" s="81" t="n"/>
-      <c r="I16" s="78" t="n"/>
+      <c r="I16" s="82" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1" s="47">
       <c r="A17" s="69" t="n"/>
       <c r="B17" s="69" t="inlineStr">
         <is>
-          <t>Маржинальность закрытых ЗН (%)</t>
+          <t>Наценка на запасные части в закрытых ЗН (%)</t>
         </is>
       </c>
       <c r="C17" s="70" t="n"/>
@@ -6520,8 +6543,8 @@
       <c r="E17" s="77" t="n"/>
       <c r="F17" s="78" t="n"/>
       <c r="G17" s="70" t="n"/>
-      <c r="H17" s="81" t="n"/>
-      <c r="I17" s="78" t="n"/>
+      <c r="H17" s="82" t="n"/>
+      <c r="I17" s="82" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1" s="47">
       <c r="A18" s="69" t="n"/>
@@ -6536,7 +6559,7 @@
       <c r="F18" s="78" t="n"/>
       <c r="G18" s="70" t="n"/>
       <c r="H18" s="81" t="n"/>
-      <c r="I18" s="78" t="n"/>
+      <c r="I18" s="82" t="n"/>
     </row>
     <row r="19" ht="33" customHeight="1" s="47">
       <c r="A19" s="69" t="n"/>
@@ -6551,7 +6574,7 @@
       <c r="F19" s="78" t="n"/>
       <c r="G19" s="70" t="n"/>
       <c r="H19" s="81" t="n"/>
-      <c r="I19" s="78" t="n"/>
+      <c r="I19" s="82" t="n"/>
     </row>
     <row r="20" ht="33" customHeight="1" s="47">
       <c r="A20" s="69" t="n"/>
@@ -6566,7 +6589,7 @@
       <c r="F20" s="78" t="n"/>
       <c r="G20" s="70" t="n"/>
       <c r="H20" s="81" t="n"/>
-      <c r="I20" s="78" t="n"/>
+      <c r="I20" s="82" t="n"/>
     </row>
     <row r="21" ht="33" customHeight="1" s="47">
       <c r="A21" s="69" t="n"/>
@@ -6581,7 +6604,7 @@
       <c r="F21" s="78" t="n"/>
       <c r="G21" s="70" t="n"/>
       <c r="H21" s="81" t="n"/>
-      <c r="I21" s="78" t="n"/>
+      <c r="I21" s="82" t="n"/>
     </row>
     <row r="22" ht="48" customHeight="1" s="47">
       <c r="A22" s="69" t="n"/>
@@ -6596,7 +6619,7 @@
       <c r="F22" s="78" t="n"/>
       <c r="G22" s="70" t="n"/>
       <c r="H22" s="81" t="n"/>
-      <c r="I22" s="78" t="n"/>
+      <c r="I22" s="82" t="n"/>
     </row>
     <row r="23" ht="48" customHeight="1" s="47">
       <c r="A23" s="69" t="n"/>
@@ -6611,7 +6634,7 @@
       <c r="F23" s="78" t="n"/>
       <c r="G23" s="70" t="n"/>
       <c r="H23" s="81" t="n"/>
-      <c r="I23" s="78" t="n"/>
+      <c r="I23" s="82" t="n"/>
     </row>
     <row r="24" ht="8" customHeight="1" s="47">
       <c r="A24" s="55" t="n"/>
@@ -6664,11 +6687,7 @@
           <t>Нч/чел.</t>
         </is>
       </c>
-      <c r="I26" s="70" t="inlineStr">
-        <is>
-          <t>Стоим. (руб.)</t>
-        </is>
-      </c>
+      <c r="I26" s="70" t="n"/>
       <c r="K26" s="43" t="n"/>
     </row>
     <row r="27" ht="33" customHeight="1" s="47">
@@ -6813,10 +6832,7 @@
       <c r="F34" s="81" t="n"/>
       <c r="G34" s="70" t="n"/>
       <c r="H34" s="81" t="n"/>
-      <c r="I34" s="81">
-        <f>SUM(I27:I33)</f>
-        <v/>
-      </c>
+      <c r="I34" s="81" t="n"/>
     </row>
     <row r="35" ht="8" customHeight="1" s="47">
       <c r="A35" s="55" t="n"/>
@@ -6928,16 +6944,14 @@
       <c r="I41" s="78" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="24">
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="A25:I25"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="A41:I41"/>
-    <mergeCell ref="H20:I20"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="D16:F16"/>
-    <mergeCell ref="H21:I21"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="D4:I4"/>
     <mergeCell ref="D37:I37"/>
@@ -6945,24 +6959,15 @@
     <mergeCell ref="D3:I3"/>
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D39:I39"/>
-    <mergeCell ref="H17:I17"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="D38:I38"/>
-    <mergeCell ref="H16:I16"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="D5:I5"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H13:I13"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="A36:I36"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="H18:I18"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="D22:F22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="H14:I14"/>
     <mergeCell ref="D21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7054,7 +7059,11 @@
     </row>
     <row r="5" ht="26" customHeight="1" s="47">
       <c r="A5" s="64" t="n"/>
-      <c r="B5" s="65" t="n"/>
+      <c r="B5" s="65" t="inlineStr">
+        <is>
+          <t>Руководитель (авто):</t>
+        </is>
+      </c>
       <c r="C5" s="64" t="n"/>
       <c r="D5" s="66" t="n"/>
       <c r="E5" s="66" t="n"/>
@@ -7536,8 +7545,8 @@
     <col width="2" customWidth="1" style="47" min="5" max="5"/>
     <col width="15" customWidth="1" style="47" min="6" max="6"/>
     <col width="2" customWidth="1" style="47" min="7" max="7"/>
-    <col width="14" customWidth="1" style="47" min="8" max="8"/>
-    <col width="16" customWidth="1" style="47" min="9" max="9"/>
+    <col width="15" customWidth="1" style="47" min="8" max="8"/>
+    <col width="12" customWidth="1" style="47" min="9" max="9"/>
     <col hidden="1" width="2" customWidth="1" style="47" min="10" max="10"/>
     <col hidden="1" width="2" customWidth="1" style="47" min="11" max="11"/>
   </cols>
@@ -7760,8 +7769,16 @@
       <c r="E13" s="77" t="n"/>
       <c r="F13" s="78" t="n"/>
       <c r="G13" s="68" t="n"/>
-      <c r="H13" s="92" t="n"/>
-      <c r="I13" s="78" t="n"/>
+      <c r="H13" s="68" t="inlineStr">
+        <is>
+          <t>vs пред. нед.</t>
+        </is>
+      </c>
+      <c r="I13" s="97" t="inlineStr">
+        <is>
+          <t>Δ %</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
       <c r="A14" s="69" t="n"/>
@@ -7775,8 +7792,8 @@
       <c r="E14" s="77" t="n"/>
       <c r="F14" s="78" t="n"/>
       <c r="G14" s="70" t="n"/>
-      <c r="H14" s="93" t="n"/>
-      <c r="I14" s="78" t="n"/>
+      <c r="H14" s="81" t="n"/>
+      <c r="I14" s="82" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1" s="47">
       <c r="A15" s="69" t="n"/>
@@ -7790,8 +7807,8 @@
       <c r="E15" s="77" t="n"/>
       <c r="F15" s="78" t="n"/>
       <c r="G15" s="70" t="n"/>
-      <c r="H15" s="93" t="n"/>
-      <c r="I15" s="78" t="n"/>
+      <c r="H15" s="81" t="n"/>
+      <c r="I15" s="82" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1" s="47">
       <c r="A16" s="69" t="n"/>
@@ -7805,14 +7822,14 @@
       <c r="E16" s="77" t="n"/>
       <c r="F16" s="78" t="n"/>
       <c r="G16" s="70" t="n"/>
-      <c r="H16" s="93" t="n"/>
-      <c r="I16" s="78" t="n"/>
+      <c r="H16" s="81" t="n"/>
+      <c r="I16" s="82" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1" s="47">
       <c r="A17" s="69" t="n"/>
       <c r="B17" s="69" t="inlineStr">
         <is>
-          <t>Маржинальность закрытых ЗН (%)</t>
+          <t>Наценка на запасные части в закрытых ЗН (%)</t>
         </is>
       </c>
       <c r="C17" s="70" t="n"/>
@@ -7820,8 +7837,8 @@
       <c r="E17" s="77" t="n"/>
       <c r="F17" s="78" t="n"/>
       <c r="G17" s="70" t="n"/>
-      <c r="H17" s="93" t="n"/>
-      <c r="I17" s="78" t="n"/>
+      <c r="H17" s="82" t="n"/>
+      <c r="I17" s="82" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1" s="47">
       <c r="A18" s="69" t="n"/>
@@ -7835,8 +7852,8 @@
       <c r="E18" s="77" t="n"/>
       <c r="F18" s="78" t="n"/>
       <c r="G18" s="70" t="n"/>
-      <c r="H18" s="93" t="n"/>
-      <c r="I18" s="78" t="n"/>
+      <c r="H18" s="81" t="n"/>
+      <c r="I18" s="82" t="n"/>
     </row>
     <row r="19" ht="33" customHeight="1" s="47">
       <c r="A19" s="69" t="n"/>
@@ -7850,8 +7867,8 @@
       <c r="E19" s="77" t="n"/>
       <c r="F19" s="78" t="n"/>
       <c r="G19" s="70" t="n"/>
-      <c r="H19" s="93" t="n"/>
-      <c r="I19" s="78" t="n"/>
+      <c r="H19" s="81" t="n"/>
+      <c r="I19" s="82" t="n"/>
     </row>
     <row r="20" ht="33" customHeight="1" s="47">
       <c r="A20" s="69" t="n"/>
@@ -7865,8 +7882,8 @@
       <c r="E20" s="77" t="n"/>
       <c r="F20" s="78" t="n"/>
       <c r="G20" s="70" t="n"/>
-      <c r="H20" s="93" t="n"/>
-      <c r="I20" s="78" t="n"/>
+      <c r="H20" s="81" t="n"/>
+      <c r="I20" s="82" t="n"/>
     </row>
     <row r="21" ht="33" customHeight="1" s="47">
       <c r="A21" s="69" t="n"/>
@@ -7880,8 +7897,8 @@
       <c r="E21" s="77" t="n"/>
       <c r="F21" s="78" t="n"/>
       <c r="G21" s="70" t="n"/>
-      <c r="H21" s="93" t="n"/>
-      <c r="I21" s="78" t="n"/>
+      <c r="H21" s="81" t="n"/>
+      <c r="I21" s="82" t="n"/>
     </row>
     <row r="22" ht="8" customHeight="1" s="47">
       <c r="A22" s="55" t="n"/>
@@ -7934,11 +7951,7 @@
           <t>Нч/чел.</t>
         </is>
       </c>
-      <c r="I24" s="70" t="inlineStr">
-        <is>
-          <t>Стоим. (руб.)</t>
-        </is>
-      </c>
+      <c r="I24" s="70" t="n"/>
     </row>
     <row r="25" ht="33" customHeight="1" s="47">
       <c r="A25" s="69" t="n"/>
@@ -8082,10 +8095,7 @@
       <c r="F32" s="81" t="n"/>
       <c r="G32" s="70" t="n"/>
       <c r="H32" s="81" t="n"/>
-      <c r="I32" s="81">
-        <f>SUM(I25:I31)</f>
-        <v/>
-      </c>
+      <c r="I32" s="81" t="n"/>
     </row>
     <row r="33" ht="8" customHeight="1" s="47">
       <c r="A33" s="55" t="n"/>
@@ -8197,14 +8207,12 @@
       <c r="I39" s="78" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="22">
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="D13:F13"/>
-    <mergeCell ref="H20:I20"/>
     <mergeCell ref="D17:F17"/>
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="D16:F16"/>
-    <mergeCell ref="H21:I21"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="D4:I4"/>
     <mergeCell ref="D37:I37"/>
@@ -8212,22 +8220,15 @@
     <mergeCell ref="A23:I23"/>
     <mergeCell ref="D3:I3"/>
     <mergeCell ref="D15:F15"/>
-    <mergeCell ref="H17:I17"/>
     <mergeCell ref="D14:F14"/>
-    <mergeCell ref="H16:I16"/>
     <mergeCell ref="D5:I5"/>
-    <mergeCell ref="H19:I19"/>
     <mergeCell ref="D35:I35"/>
     <mergeCell ref="A39:I39"/>
     <mergeCell ref="A34:I34"/>
-    <mergeCell ref="H13:I13"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="D19:F19"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="H18:I18"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="D36:I36"/>
-    <mergeCell ref="H14:I14"/>
     <mergeCell ref="D21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Widen daily shop pipeline value column
</commit_message>
<xml_diff>
--- a/backend/templates/report_template.xlsx
+++ b/backend/templates/report_template.xlsx
@@ -5918,13 +5918,9 @@
         </is>
       </c>
       <c r="E12" s="77" t="n"/>
-      <c r="F12" s="78" t="n"/>
-      <c r="G12" s="68" t="n"/>
-      <c r="H12" s="68" t="inlineStr">
-        <is>
-          <t>Норма</t>
-        </is>
-      </c>
+      <c r="F12" s="77" t="n"/>
+      <c r="G12" s="77" t="n"/>
+      <c r="H12" s="77" t="n"/>
       <c r="I12" s="78" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1" s="47">
@@ -5937,9 +5933,9 @@
       <c r="C13" s="70" t="n"/>
       <c r="D13" s="81" t="n"/>
       <c r="E13" s="77" t="n"/>
-      <c r="F13" s="78" t="n"/>
-      <c r="G13" s="70" t="n"/>
-      <c r="H13" s="81" t="n"/>
+      <c r="F13" s="77" t="n"/>
+      <c r="G13" s="77" t="n"/>
+      <c r="H13" s="77" t="n"/>
       <c r="I13" s="78" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
@@ -5952,9 +5948,9 @@
       <c r="C14" s="70" t="n"/>
       <c r="D14" s="81" t="n"/>
       <c r="E14" s="77" t="n"/>
-      <c r="F14" s="78" t="n"/>
-      <c r="G14" s="70" t="n"/>
-      <c r="H14" s="81" t="n"/>
+      <c r="F14" s="77" t="n"/>
+      <c r="G14" s="77" t="n"/>
+      <c r="H14" s="77" t="n"/>
       <c r="I14" s="78" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1" s="47">
@@ -5967,13 +5963,9 @@
       <c r="C15" s="70" t="n"/>
       <c r="D15" s="81" t="n"/>
       <c r="E15" s="77" t="n"/>
-      <c r="F15" s="78" t="n"/>
-      <c r="G15" s="70" t="n"/>
-      <c r="H15" s="70" t="inlineStr">
-        <is>
-          <t>Цель: 0</t>
-        </is>
-      </c>
+      <c r="F15" s="77" t="n"/>
+      <c r="G15" s="77" t="n"/>
+      <c r="H15" s="77" t="n"/>
       <c r="I15" s="78" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1" s="47">
@@ -5986,13 +5978,9 @@
       <c r="C16" s="70" t="n"/>
       <c r="D16" s="81" t="n"/>
       <c r="E16" s="77" t="n"/>
-      <c r="F16" s="78" t="n"/>
-      <c r="G16" s="70" t="n"/>
-      <c r="H16" s="70" t="inlineStr">
-        <is>
-          <t>Цель: 0</t>
-        </is>
-      </c>
+      <c r="F16" s="77" t="n"/>
+      <c r="G16" s="77" t="n"/>
+      <c r="H16" s="77" t="n"/>
       <c r="I16" s="78" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1" s="47">
@@ -6005,9 +5993,9 @@
       <c r="C17" s="70" t="n"/>
       <c r="D17" s="81" t="n"/>
       <c r="E17" s="77" t="n"/>
-      <c r="F17" s="78" t="n"/>
-      <c r="G17" s="70" t="n"/>
-      <c r="H17" s="81" t="n"/>
+      <c r="F17" s="77" t="n"/>
+      <c r="G17" s="77" t="n"/>
+      <c r="H17" s="77" t="n"/>
       <c r="I17" s="78" t="n"/>
     </row>
     <row r="18" ht="8" customHeight="1" s="47">
@@ -6208,27 +6196,21 @@
       <c r="I27" s="78" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="D13:F13"/>
+  <mergeCells count="14">
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="D17:I17"/>
     <mergeCell ref="A27:I27"/>
-    <mergeCell ref="D17:F17"/>
-    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D16:I16"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="D4:I4"/>
-    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="D12:I12"/>
     <mergeCell ref="D3:I3"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="D15:I15"/>
     <mergeCell ref="A19:I19"/>
-    <mergeCell ref="H16:I16"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="D14:I14"/>
     <mergeCell ref="A11:I11"/>
-    <mergeCell ref="H15:I15"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A6:I6"/>
-    <mergeCell ref="H14:I14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>
@@ -6966,8 +6948,8 @@
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="A36:I36"/>
+    <mergeCell ref="D22:F22"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="D22:F22"/>
     <mergeCell ref="D21:F21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7224,9 +7206,9 @@
         </is>
       </c>
       <c r="E13" s="77" t="n"/>
-      <c r="F13" s="78" t="n"/>
-      <c r="G13" s="68" t="n"/>
-      <c r="H13" s="92" t="n"/>
+      <c r="F13" s="77" t="n"/>
+      <c r="G13" s="77" t="n"/>
+      <c r="H13" s="77" t="n"/>
       <c r="I13" s="78" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1" s="47">
@@ -7239,9 +7221,9 @@
       <c r="C14" s="70" t="n"/>
       <c r="D14" s="81" t="n"/>
       <c r="E14" s="77" t="n"/>
-      <c r="F14" s="78" t="n"/>
-      <c r="G14" s="70" t="n"/>
-      <c r="H14" s="93" t="n"/>
+      <c r="F14" s="77" t="n"/>
+      <c r="G14" s="77" t="n"/>
+      <c r="H14" s="77" t="n"/>
       <c r="I14" s="78" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1" s="47">
@@ -7254,9 +7236,9 @@
       <c r="C15" s="70" t="n"/>
       <c r="D15" s="81" t="n"/>
       <c r="E15" s="77" t="n"/>
-      <c r="F15" s="78" t="n"/>
-      <c r="G15" s="70" t="n"/>
-      <c r="H15" s="93" t="n"/>
+      <c r="F15" s="77" t="n"/>
+      <c r="G15" s="77" t="n"/>
+      <c r="H15" s="77" t="n"/>
       <c r="I15" s="78" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1" s="47">
@@ -7269,9 +7251,9 @@
       <c r="C16" s="70" t="n"/>
       <c r="D16" s="81" t="n"/>
       <c r="E16" s="77" t="n"/>
-      <c r="F16" s="78" t="n"/>
-      <c r="G16" s="70" t="n"/>
-      <c r="H16" s="94" t="n"/>
+      <c r="F16" s="77" t="n"/>
+      <c r="G16" s="77" t="n"/>
+      <c r="H16" s="77" t="n"/>
       <c r="I16" s="78" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1" s="47">
@@ -7284,9 +7266,9 @@
       <c r="C17" s="70" t="n"/>
       <c r="D17" s="81" t="n"/>
       <c r="E17" s="77" t="n"/>
-      <c r="F17" s="78" t="n"/>
-      <c r="G17" s="70" t="n"/>
-      <c r="H17" s="94" t="n"/>
+      <c r="F17" s="77" t="n"/>
+      <c r="G17" s="77" t="n"/>
+      <c r="H17" s="77" t="n"/>
       <c r="I17" s="78" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1" s="47">
@@ -7299,9 +7281,9 @@
       <c r="C18" s="70" t="n"/>
       <c r="D18" s="81" t="n"/>
       <c r="E18" s="77" t="n"/>
-      <c r="F18" s="78" t="n"/>
-      <c r="G18" s="70" t="n"/>
-      <c r="H18" s="93" t="n"/>
+      <c r="F18" s="77" t="n"/>
+      <c r="G18" s="77" t="n"/>
+      <c r="H18" s="77" t="n"/>
       <c r="I18" s="78" t="n"/>
     </row>
     <row r="19" ht="8" customHeight="1" s="47">
@@ -7502,27 +7484,21 @@
       <c r="I28" s="78" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="D17:F17"/>
+  <mergeCells count="14">
+    <mergeCell ref="D13:I13"/>
+    <mergeCell ref="D17:I17"/>
     <mergeCell ref="A12:I12"/>
-    <mergeCell ref="D16:F16"/>
+    <mergeCell ref="D16:I16"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="D4:I4"/>
-    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="D18:I18"/>
     <mergeCell ref="D3:I3"/>
-    <mergeCell ref="D15:F15"/>
     <mergeCell ref="A20:I20"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="D15:I15"/>
     <mergeCell ref="A28:I28"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="D14:I14"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A6:I6"/>
-    <mergeCell ref="H14:I14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>